<commit_message>
Bang ID Chuong 2 (docs/bang_ID_L10_C2.xlsx) cap nhat theo ID moi diem thuoc mien nghiem
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SrV2RdTxyMnQTjbX6LNoBV
</commit_message>
<xml_diff>
--- a/docs/bang_ID_L10_C2.xlsx
+++ b/docs/bang_ID_L10_C2.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Huong dan" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ID Chuong 2'!$A$1:$N$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ID Chuong 2'!$A$1:$N$59</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N53"/>
+  <dimension ref="A1:N59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -563,17 +563,17 @@
       <c r="G2" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Nhận ra bất phương trình bậc nhất hai ẩn trong các biểu thức cho trước</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n"/>
       <c r="M2" s="2" t="n"/>
-      <c r="N2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -583,7 +583,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>023</t>
+          <t>025</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -603,23 +603,39 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B3_NB023_MC_A</t>
+          <t>L10_C2_B3_NB025_MC_A</t>
         </is>
       </c>
       <c r="G3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="n"/>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>cua_hang_but, xuong_may, cho_hang, protein_thit_ca, cuoc_dien_thoai, lam_them, thue_o_to</t>
+        </is>
+      </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Kiểm tra một cặp số có phải nghiệm của bất phương trình không</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr"/>
-      <c r="L3" s="2" t="inlineStr"/>
-      <c r="M3" s="2" t="n"/>
-      <c r="N3" s="2" t="inlineStr"/>
+          <t>Chọn bất phương trình mô tả đúng tình huống thực tế</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Chọn bất phương trình mô tả đúng một tình huống thực tế.</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>09/10/2026 sang loc cau thuc te chuong 2: them boi_canh</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Toán thực tế ở mức NB (quy tắc: thực tế không có NB/TH trừ Đ/S rất dễ) - cần nâng VD/VDC hoặc giữ nếu cô duyệt; Bối cảnh dùng chung với YCCĐ/TF khác: 028</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -629,7 +645,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>023</t>
+          <t>024</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -639,41 +655,45 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>SA</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B3_NB023_SA_A</t>
+          <t>L10_C2_B3_NB024_MC_B</t>
         </is>
       </c>
       <c r="G4" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="n"/>
+      <c r="I4" s="2" t="n"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Kiểm tra một cặp số có phải nghiệm của bất phương trình không</t>
+          <t>Đọc hình miền nghiệm của một bất phương trình (đề không cho bất phương trình): xác định điểm thuộc miền nghiệm (điểm trên bờ nét liền thì thuộc, nét đứt thì không)</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trả lời ngắn: cho một bất phương trình bậc nhất hai ẩn và $5$ cặp số, ĐẾM số cặp số là nghiệm. (cùng dạng với NB023_MC_A: kiểm tra một cặp số có phải nghiệm của bất phương trình không.) Số cặp là nghiệm chọn trước trong </t>
+          <t>Đọc HÌNH miền nghiệm của một bất phương trình bậc nhất hai ẩn (không cho bất phương trình): điểm nào thuộc miền nghiệm. Nhiễu: điểm ở phần bị gạch, điểm trên bờ vẽ nét đứt.</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>CLAUDE THEM 15/10/2026 - ban tra loi ngan cua NB023_MC_A (cung Dang): dem so cap so la nghiem trong 5 cap so; co Lan duyet lai</t>
-        </is>
-      </c>
-      <c r="M4" s="2" t="n"/>
-      <c r="N4" s="2" t="inlineStr"/>
+          <t>CLAUDE THEM 15/10/2026 - co Lan duyet ke hoach ID (diem thuoc mien nghiem; co Lan: dung hinh thi chi la NB); hoi diem nao thuoc mien nghiem; khac NB023 (NB023 c</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>Mới 15/10/2026 (dạng điểm thuộc miền nghiệm, ID cô Lan đặt)</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -683,7 +703,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>025</t>
+          <t>024</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -693,49 +713,45 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>MC</t>
+          <t>SA</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B3_NB025_MC_A</t>
+          <t>L10_C2_B3_NB024_SA_B</t>
         </is>
       </c>
       <c r="G5" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="H5" s="2" t="inlineStr"/>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>cua_hang_but, xuong_may, cho_hang, protein_thit_ca, cuoc_dien_thoai, lam_them, thue_o_to</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="H5" s="2" t="n"/>
+      <c r="I5" s="2" t="n"/>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Chọn bất phương trình mô tả đúng tình huống thực tế</t>
+          <t>Đọc hình miền nghiệm của một bất phương trình (đề không cho bất phương trình): xác định điểm thuộc miền nghiệm (điểm trên bờ nét liền thì thuộc, nét đứt thì không)</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Chọn bất phương trình mô tả đúng một tình huống thực tế.</t>
+          <t>Đọc HÌNH miền nghiệm của một bất phương trình bậc nhất hai ẩn: trong $5$ điểm, có bao nhiêu điểm thuộc miền nghiệm. Số điểm thuộc chọn trước trong $\{1; 2; 3; 4\}$; thường có một điểm nằm trên bờ (nét liền thì thuộc, nét</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>09/10/2026 sang loc cau thuc te chuong 2: them boi_canh</t>
-        </is>
-      </c>
-      <c r="M5" s="3" t="inlineStr">
-        <is>
-          <t>Toán thực tế ở mức NB (quy tắc: thực tế không có NB/TH trừ Đ/S rất dễ) - cần nâng VD/VDC hoặc giữ nếu cô duyệt; Bối cảnh dùng chung với YCCĐ/TF khác: 028</t>
-        </is>
-      </c>
-      <c r="N5" s="2" t="inlineStr"/>
+          <t>CLAUDE THEM 15/10/2026 - co Lan duyet ke hoach ID (diem thuoc mien nghiem; co Lan: dung hinh thi chi la NB); ban tra loi ngan cua TH024_MC_B (cung Dang): dem so</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>Mới 15/10/2026 (dạng điểm thuộc miền nghiệm, ID cô Lan đặt)</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -771,8 +787,8 @@
       <c r="G6" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H6" s="2" t="inlineStr"/>
-      <c r="I6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="n"/>
+      <c r="I6" s="2" t="n"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
           <t>Chọn hình vẽ đúng của miền nghiệm</t>
@@ -783,9 +799,9 @@
           <t>Chọn hình biểu diễn miền nghiệm - bờ $d$ cắt hai trục tại $(p; 0)$, $(0; q)$.</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="n"/>
       <c r="M6" s="2" t="n"/>
-      <c r="N6" s="2" t="inlineStr"/>
+      <c r="N6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -805,97 +821,109 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>TL</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B3_TH024_TL_A</t>
+          <t>L10_C2_B3_TH024_MC_B</t>
         </is>
       </c>
       <c r="G7" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H7" s="2" t="inlineStr"/>
-      <c r="I7" s="2" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="H7" s="2" t="n"/>
+      <c r="I7" s="2" t="n"/>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Biểu diễn miền nghiệm trên mặt phẳng toạ độ</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>Tự luận: các bước vẽ miền nghiệm - tìm hai giao điểm của đường bờ với hai trục.</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="inlineStr"/>
-      <c r="M7" s="2" t="n"/>
-      <c r="N7" s="2" t="inlineStr"/>
+          <t>Cho bất phương trình, kiểm tra một điểm (cặp số) có thuộc miền nghiệm (là nghiệm) của bất phương trình không</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="n"/>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>DOI ID 15/10/2026 (co Lan): L10_C2_B3_NB023_MC_A -&gt; L10_C2_B3_TH024_MC_B; cho bat phuong trinh xet diem thuoc mien nghiem la muc TH, 023 danh cho tinh F(x;y)</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>Đổi ID 15/10/2026 (cô Lan) từ L10_C2_B3_NB023_MC_A</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>B4</t>
+          <t>B3</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>026</t>
+          <t>024</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>NB</t>
+          <t>TH</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>MC</t>
+          <t>SA</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_NB026_MC_A</t>
+          <t>L10_C2_B3_TH024_SA_B</t>
         </is>
       </c>
       <c r="G8" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="H8" s="2" t="inlineStr"/>
-      <c r="I8" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H8" s="2" t="n"/>
+      <c r="I8" s="2" t="n"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Nhận ra hệ bất phương trình bậc nhất hai ẩn</t>
+          <t>Cho bất phương trình, kiểm tra một điểm (cặp số) có thuộc miền nghiệm (là nghiệm) của bất phương trình không</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Nhận ra hệ bất phương trình bậc nhất hai ẩn.</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr"/>
-      <c r="M8" s="2" t="n"/>
-      <c r="N8" s="2" t="inlineStr"/>
+          <t>Trả lời ngắn: cho một bất phương trình bậc nhất hai ẩn và $5$ cặp số, ĐẾM số cặp số là nghiệm. (cùng dạng với TH024_MC_B: kiểm tra một cặp số có phải nghiệm của bất phương trình không; trước 15/10/2026 là NB023_SA_A.) Số</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>CLAUDE THEM 15/10/2026 - ban tra loi ngan cua NB023_MC_A (cung Dang): dem so cap so la nghiem trong 5 cap so; co Lan duyet lai; DOI ID 15/10/2026 (co Lan): L10_</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>Đổi ID 15/10/2026 (cô Lan) từ L10_C2_B3_NB023_SA_A</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>B4</t>
+          <t>B3</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>027</t>
+          <t>024</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -905,7 +933,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>MC</t>
+          <t>TL</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -915,23 +943,27 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_TH027_MC_A</t>
+          <t>L10_C2_B3_TH024_TL_A</t>
         </is>
       </c>
       <c r="G9" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H9" s="2" t="inlineStr"/>
-      <c r="I9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="n"/>
+      <c r="I9" s="2" t="n"/>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Chọn hình vẽ đúng của miền nghiệm hệ</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr"/>
-      <c r="L9" s="2" t="inlineStr"/>
+          <t>Biểu diễn miền nghiệm trên mặt phẳng toạ độ</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Tự luận: các bước vẽ miền nghiệm - tìm hai giao điểm của đường bờ với hai trục.</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="n"/>
       <c r="M9" s="2" t="n"/>
-      <c r="N9" s="2" t="inlineStr"/>
+      <c r="N9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -941,17 +973,17 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>027</t>
+          <t>026</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>TH</t>
+          <t>NB</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>TL</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -961,27 +993,27 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_TH027_TL_A</t>
+          <t>L10_C2_B4_NB026_MC_A</t>
         </is>
       </c>
       <c r="G10" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H10" s="2" t="inlineStr"/>
-      <c r="I10" s="2" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="H10" s="2" t="n"/>
+      <c r="I10" s="2" t="n"/>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Biểu diễn miền nghiệm của hệ trên mặt phẳng toạ độ</t>
+          <t>Nhận ra hệ bất phương trình bậc nhất hai ẩn</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Tự luận: miền nghiệm của hệ là tam giác vuông - tìm đỉnh và tính diện tích.</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="inlineStr"/>
+          <t>Nhận ra hệ bất phương trình bậc nhất hai ẩn.</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="n"/>
       <c r="M10" s="2" t="n"/>
-      <c r="N10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -991,12 +1023,12 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>028</t>
+          <t>027</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>VD</t>
+          <t>TH</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -1011,23 +1043,23 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_VD028_MC_A</t>
+          <t>L10_C2_B4_TH027_MC_A</t>
         </is>
       </c>
       <c r="G11" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="H11" s="2" t="inlineStr"/>
-      <c r="I11" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H11" s="2" t="n"/>
+      <c r="I11" s="2" t="n"/>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Tìm giá trị lớn nhất, nhỏ nhất của F = ax + by trên miền đa giác</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr"/>
-      <c r="L11" s="2" t="inlineStr"/>
+          <t>Chọn hình vẽ đúng của miền nghiệm hệ</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="n"/>
+      <c r="L11" s="2" t="n"/>
       <c r="M11" s="2" t="n"/>
-      <c r="N11" s="2" t="inlineStr"/>
+      <c r="N11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1037,51 +1069,55 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>028</t>
+          <t>027</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>VD</t>
+          <t>TH</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>SA</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_VD028_SA_A</t>
+          <t>L10_C2_B4_TH027_MC_B</t>
         </is>
       </c>
       <c r="G12" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="H12" s="2" t="inlineStr"/>
-      <c r="I12" s="2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="2" t="n"/>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Tìm giá trị lớn nhất, nhỏ nhất của F = ax + by trên miền đa giác</t>
+          <t>Đọc hình miền nghiệm của hệ bất phương trình (đề không cho hệ): xác định điểm thuộc miền nghiệm (điểm trên bờ nét liền thì thuộc, nét đứt thì không)</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Trả lời ngắn: giá trị lớn nhất của F = px + qy trên miền nghiệm của hệ.</t>
+          <t>Đọc HÌNH miền nghiệm của một HỆ hai bất phương trình bậc nhất hai ẩn (không cho hệ): điểm nào thuộc miền nghiệm. Nhiễu ưu tiên điểm chỉ vi phạm một bất phương trình (nằm ở phần bị gạch bởi một bờ, hoặc trên bờ nét đứt).</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>15/10/2026 co Lan duyet: thong nhat Dang voi VD028_MC_A (cung dang: tim gia tri lon nhat/nho nhat cua F = ax + by tren mien da giac)</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="n"/>
-      <c r="N12" s="2" t="inlineStr"/>
+          <t>CLAUDE THEM 15/10/2026 - co Lan chot ID TH027_MC_B (hinh ve he, diem thuoc khong); hoi diem nao thuoc mien nghiem; co Lan duyet lai noi dung</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>Mới 15/10/2026 (dạng điểm thuộc miền nghiệm, ID cô Lan đặt)</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1091,143 +1127,151 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
+          <t>027</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>TH</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>SA</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>L10_C2_B4_TH027_SA_B</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="n"/>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Đọc hình miền nghiệm của hệ bất phương trình (đề không cho hệ): xác định điểm thuộc miền nghiệm (điểm trên bờ nét liền thì thuộc, nét đứt thì không)</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Đọc HÌNH miền nghiệm của một HỆ hai bất phương trình: trong $5$ điểm, có bao nhiêu điểm thuộc miền nghiệm. Số điểm thuộc chọn trước trong $\{1; 2; 3; 4\}$.</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CLAUDE THEM 15/10/2026 - co Lan chot ID TH027_MC_B (hinh ve he, diem thuoc khong); ban tra loi ngan cua TH027_MC_B (cung Dang): dem so diem thuoc trong 5 diem; </t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>Mới 15/10/2026 (dạng điểm thuộc miền nghiệm, ID cô Lan đặt)</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>B4</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>027</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>TH</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>L10_C2_B4_TH027_TL_A</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" s="2" t="n"/>
+      <c r="I14" s="2" t="n"/>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Biểu diễn miền nghiệm của hệ trên mặt phẳng toạ độ</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Tự luận: miền nghiệm của hệ là tam giác vuông - tìm đỉnh và tính diện tích.</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="n"/>
+      <c r="M14" s="2" t="n"/>
+      <c r="N14" s="2" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>B4</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
           <t>028</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>VD</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>TL</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>MC</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>L10_C2_B4_VD028_TL_A</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="n">
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>L10_C2_B4_VD028_MC_A</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H13" s="2" t="inlineStr"/>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>xuong_san_xuat, xuong_may, nong_dan_ngo_khoai, tiem_banh, trai_ga, bep_an_rau</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>Bài toán tối ưu thực tiễn dẫn đến hệ bất phương trình</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>Tự luận: bài toán tối ưu thực tiễn dẫn đến hệ bất phương trình.</t>
-        </is>
-      </c>
-      <c r="L13" s="2" t="inlineStr">
-        <is>
-          <t>09/10/2026 sang loc cau thuc te chuong 2: them boi_canh</t>
-        </is>
-      </c>
-      <c r="M13" s="3" t="inlineStr">
-        <is>
-          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025</t>
-        </is>
-      </c>
-      <c r="N13" s="2" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr"/>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>(cả chương)</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr"/>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>TF</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>L10_C2_TF_A</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="H14" s="2" t="inlineStr"/>
-      <c r="I14" s="2" t="inlineStr"/>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>Câu dẫn là bất phương trình bậc nhất 2 ẩn</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
-          <t>Đúng/Sai - bất phương trình bậc nhất hai ẩn (bản nháp phát triển).</t>
-        </is>
-      </c>
-      <c r="L14" s="2" t="inlineStr"/>
-      <c r="M14" s="2" t="n"/>
-      <c r="N14" s="2" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr"/>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>(cả chương)</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr"/>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>TF</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>L10_C2_TF_B</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H15" s="2" t="inlineStr"/>
-      <c r="I15" s="2" t="inlineStr"/>
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="n"/>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>Câu dẫn là hệ bất phương trình bậc nhất 2 ẩn</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>Đúng/Sai - hệ bất phương trình bậc nhất hai ẩn $x \ge 0$, $y \ge 0$ và hai bất phương trình khác (miền nghiệm là tứ giác nguyên đỉnh) kèm biểu thức $F = px + qy$.</t>
-        </is>
-      </c>
-      <c r="L15" s="2" t="inlineStr"/>
+          <t>Tìm giá trị lớn nhất, nhỏ nhất của F = ax + by trên miền đa giác</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="n"/>
+      <c r="L15" s="2" t="n"/>
       <c r="M15" s="2" t="n"/>
-      <c r="N15" s="2" t="inlineStr"/>
+      <c r="N15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1237,47 +1281,51 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>027</t>
+          <t>028</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>TH</t>
+          <t>VD</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>MC</t>
+          <t>SA</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_TH027_MC_B</t>
+          <t>L10_C2_B4_VD028_SA_A</t>
         </is>
       </c>
       <c r="G16" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H16" s="2" t="inlineStr"/>
-      <c r="I16" s="2" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="n"/>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Miền nghiệm của hệ là đa giác gì (tam giác, tứ giác, ngũ giác...)</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr"/>
+          <t>Tìm giá trị lớn nhất, nhỏ nhất của F = ax + by trên miền đa giác</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Trả lời ngắn: giá trị lớn nhất của F = px + qy trên miền nghiệm của hệ.</t>
+        </is>
+      </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>CLAUDE THEM 29/09/2026 - co Lan kiem tra lai ID va mo ta</t>
+          <t>15/10/2026 co Lan duyet: thong nhat Dang voi VD028_MC_A (cung dang: tim gia tri lon nhat/nho nhat cua F = ax + by tren mien da giac)</t>
         </is>
       </c>
       <c r="M16" s="2" t="n"/>
-      <c r="N16" s="2" t="inlineStr"/>
+      <c r="N16" s="2" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1287,174 +1335,158 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>027</t>
+          <t>028</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>TH</t>
+          <t>VD</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>SA</t>
+          <t>TL</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>L10_C2_B4_VD028_TL_A</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>xuong_san_xuat, xuong_may, nong_dan_ngo_khoai, tiem_banh, trai_ga, bep_an_rau</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Bài toán tối ưu thực tiễn dẫn đến hệ bất phương trình</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Tự luận: bài toán tối ưu thực tiễn dẫn đến hệ bất phương trình.</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>09/10/2026 sang loc cau thuc te chuong 2: them boi_canh</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n"/>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>(cả chương)</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="n"/>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>TF</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>L10_C2_TF_A</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H18" s="2" t="n"/>
+      <c r="I18" s="2" t="n"/>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Câu dẫn là bất phương trình bậc nhất 2 ẩn</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Đúng/Sai - bất phương trình bậc nhất hai ẩn (bản nháp phát triển).</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="n"/>
+      <c r="M18" s="2" t="n"/>
+      <c r="N18" s="2" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n"/>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>(cả chương)</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="n"/>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>TF</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
           <t>B</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>L10_C2_B4_TH027_SA_B</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H17" s="2" t="inlineStr"/>
-      <c r="I17" s="2" t="inlineStr"/>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>Miền nghiệm của hệ là đa giác gì (tam giác, tứ giác, ngũ giác...)</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>Trả lời ngắn: miền nghiệm của hệ (hình chữ nhật cắt bởi một nửa mặt phẳng) là đa giác có bao nhiêu ĐỈNH (hoặc CẠNH). (cùng dạng với TH027_MC_B: miền nghiệm của hệ là đa giác gì: tam giác, tứ giác, ngũ giác.) Số đỉnh = số</t>
-        </is>
-      </c>
-      <c r="L17" s="2" t="inlineStr">
-        <is>
-          <t>CLAUDE THEM 15/10/2026 - ban tra loi ngan cua TH027_MC_B (cung Dang): mien nghiem la da giac co bao nhieu dinh (canh); co Lan duyet lai</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="n"/>
-      <c r="N17" s="2" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>B3</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>023</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>NB</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>SA</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>L10_C2_B3_NB023_SA_B</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H18" s="2" t="inlineStr"/>
-      <c r="I18" s="2" t="inlineStr"/>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>Cho bất phương trình ax + by ≤ c (hoặc ≥, &lt;, &gt;) và một nghiệm nguyên M thuộc miền nghiệm: tính giá trị biểu thức F(x; y) = ax + by tại M</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>Trả lời ngắn: tính giá trị $F\left(x; y\right) = ax + by$ (đúng DẠNG này, không có hằng số) tại một nghiệm nguyên $M$ của bất phương trình $ax + by \;\square\; c$ (cùng $a$, $b$ với vế trái).</t>
-        </is>
-      </c>
-      <c r="L18" s="2" t="inlineStr">
-        <is>
-          <t>CLAUDE THEM 29/09/2026 - co Lan kiem tra lai ID va mo ta; 12/10/2026 co Lan: F chi co dang ax + by, M phai thuoc mien nghiem (chon ngau nhien nghiem nguyen); 15</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="n"/>
-      <c r="N18" s="2" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>B3</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>023</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>NB</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>MC</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B3_NB023_MC_B</t>
+          <t>L10_C2_TF_B</t>
         </is>
       </c>
       <c r="G19" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H19" s="2" t="inlineStr"/>
-      <c r="I19" s="2" t="inlineStr"/>
+      <c r="H19" s="2" t="n"/>
+      <c r="I19" s="2" t="n"/>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>Cho bất phương trình ax + by ≤ c (hoặc ≥, &lt;, &gt;) và một nghiệm nguyên M thuộc miền nghiệm: tính giá trị biểu thức F(x; y) = ax + by tại M</t>
+          <t>Câu dẫn là hệ bất phương trình bậc nhất 2 ẩn</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>Trắc nghiệm cùng dạng với NB023_SA_B_01: tính $F\left(x; y\right) = ax + by$ tại một nghiệm nguyên $M$.</t>
-        </is>
-      </c>
-      <c r="L19" s="2" t="inlineStr">
-        <is>
-          <t>CLAUDE THEM 15/10/2026 - ban trac nghiem cua NB023_SA_B (cung Dang): tinh F = ax + by tai nghiem nguyen M; co Lan duyet lai</t>
-        </is>
-      </c>
+          <t>Đúng/Sai - hệ bất phương trình bậc nhất hai ẩn $x \ge 0$, $y \ge 0$ và hai bất phương trình khác (miền nghiệm là tứ giác nguyên đỉnh) kèm biểu thức $F = px + qy$.</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="n"/>
       <c r="M19" s="2" t="n"/>
-      <c r="N19" s="2" t="inlineStr"/>
+      <c r="N19" s="2" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>B4</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>025</t>
+          <t>027</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>NB</t>
+          <t>TH</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1464,44 +1496,36 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B3_NB025_MC_B</t>
+          <t>L10_C2_B4_TH027_MC_C</t>
         </is>
       </c>
       <c r="G20" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="H20" s="2" t="inlineStr"/>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>pha_che</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="H20" s="2" t="n"/>
+      <c r="I20" s="2" t="n"/>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>Bài toán thực tiễn pha chế nước giải khát: lập bất phương trình, hệ bất phương trình và tìm phương án có điểm thưởng cao nhất (ba điều kiện)</t>
-        </is>
-      </c>
-      <c r="K20" s="2" t="inlineStr">
-        <is>
-          <t>Pha chế: bất phương trình về lượng ĐƯỜNG.</t>
-        </is>
-      </c>
+          <t>Miền nghiệm của hệ là đa giác gì (tam giác, tứ giác, ngũ giác...)</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="n"/>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 1: pha che nuoc); boi_canh pha_che; so lieu ngau nhien cung cau truc</t>
-        </is>
-      </c>
-      <c r="M20" s="3" t="inlineStr">
-        <is>
-          <t>Toán thực tế ở mức NB (quy tắc: thực tế không có NB/TH trừ Đ/S rất dễ) - cần nâng VD/VDC hoặc giữ nếu cô duyệt; Bối cảnh dùng chung với YCCĐ/TF khác: 028, TF</t>
-        </is>
-      </c>
-      <c r="N20" s="2" t="inlineStr"/>
+          <t>CLAUDE THEM 29/09/2026 - co Lan kiem tra lai ID va mo ta; DOI ID 15/10/2026 (co Lan): chu B -&gt; C de chu B danh cho dang diem thuoc mien nghiem</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>Đổi ID 15/10/2026 (cô Lan) từ L10_C2_B4_TH027_MC_B</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1511,59 +1535,55 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>028</t>
+          <t>027</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>VD</t>
+          <t>TH</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>MC</t>
+          <t>SA</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_VD028_MC_B</t>
+          <t>L10_C2_B4_TH027_SA_C</t>
         </is>
       </c>
       <c r="G21" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="H21" s="2" t="inlineStr"/>
-      <c r="I21" s="2" t="inlineStr">
-        <is>
-          <t>pha_che</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="H21" s="2" t="n"/>
+      <c r="I21" s="2" t="n"/>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>Bài toán thực tiễn pha chế nước giải khát: lập bất phương trình, hệ bất phương trình và tìm phương án có điểm thưởng cao nhất (ba điều kiện)</t>
+          <t>Miền nghiệm của hệ là đa giác gì (tam giác, tứ giác, ngũ giác...)</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>Pha chế: chọn hệ bất phương trình mô tả đúng các điều kiện.</t>
+          <t>Trả lời ngắn: miền nghiệm của hệ (hình chữ nhật cắt bởi một nửa mặt phẳng) là đa giác có bao nhiêu ĐỈNH (hoặc CẠNH). (cùng dạng với TH027_MC_C: miền nghiệm của hệ là đa giác gì: tam giác, tứ giác, ngũ giác; trước 15/10/2</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 1: pha che nuoc); boi_canh pha_che; so lieu ngau nhien cung cau truc</t>
-        </is>
-      </c>
-      <c r="M21" s="3" t="inlineStr">
-        <is>
-          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF; Cùng chữ "Dang" với các chữ B/C (MC/SA) của VD028: cùng dạng nhưng nhiều chữ (khác bối cảnh hoặc khác mức)</t>
-        </is>
-      </c>
-      <c r="N21" s="2" t="inlineStr"/>
+          <t>CLAUDE THEM 15/10/2026 - ban tra loi ngan cua TH027_MC_B (cung Dang): mien nghiem la da giac co bao nhieu dinh (canh); co Lan duyet lai; DOI ID 15/10/2026 (co L</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>Đổi ID 15/10/2026 (cô Lan) từ L10_C2_B4_TH027_SA_B</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1573,7 +1593,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>028</t>
+          <t>027</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1583,7 +1603,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>SA</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1593,39 +1613,35 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_VD028_SA_B</t>
+          <t>L10_C2_B4_VD027_MC_B</t>
         </is>
       </c>
       <c r="G22" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="H22" s="2" t="inlineStr"/>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>pha_che</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="H22" s="2" t="n"/>
+      <c r="I22" s="2" t="n"/>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>Bài toán thực tiễn pha chế nước giải khát: lập bất phương trình, hệ bất phương trình và tìm phương án có điểm thưởng cao nhất (ba điều kiện)</t>
+          <t>Cho hệ bất phương trình bậc nhất hai ẩn, kiểm tra điểm thuộc miền nghiệm (thay toạ độ vào tất cả các bất phương trình của hệ) - mức Vận dụng, ngoài YCCĐ</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>Pha chế (VD): số đỉnh của miền nghiệm.</t>
+          <t>Cho hệ $2$ hoặc $3$ bất phương trình bậc nhất hai ẩn: điểm nào thuộc miền nghiệm của hệ. Nhiễu ưu tiên điểm thoả mãn mọi bất phương trình trừ một.</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 1: pha che nuoc); boi_canh pha_che; so lieu ngau nhien cung cau truc</t>
-        </is>
-      </c>
-      <c r="M22" s="3" t="inlineStr">
-        <is>
-          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF; Cùng chữ "Dang" với các chữ B/C (MC/SA) của VD028: cùng dạng nhưng nhiều chữ (khác bối cảnh hoặc khác mức)</t>
-        </is>
-      </c>
-      <c r="N22" s="2" t="inlineStr"/>
+          <t>LUYEN TAP THEM - MUC VAN DUNG CAO HON YCCD TH027 CUA BO; CLAUDE THEM 15/10/2026 - co Lan duyet ke hoach ID (diem thuoc mien nghiem cua he; co Lan: he bat phuong</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>Mới 15/10/2026 (dạng điểm thuộc miền nghiệm, ID cô Lan đặt); Luyện tập thêm (ngoài YCCĐ)</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1635,7 +1651,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>028</t>
+          <t>027</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -1645,68 +1661,60 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>MC</t>
+          <t>SA</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_VD028_MC_C</t>
+          <t>L10_C2_B4_VD027_SA_B</t>
         </is>
       </c>
       <c r="G23" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="H23" s="2" t="inlineStr">
-        <is>
-          <t>VDC</t>
-        </is>
-      </c>
-      <c r="I23" s="2" t="inlineStr">
-        <is>
-          <t>pha_che</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="H23" s="2" t="n"/>
+      <c r="I23" s="2" t="n"/>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>Bài toán thực tiễn pha chế nước giải khát: lập bất phương trình, hệ bất phương trình và tìm phương án có điểm thưởng cao nhất (ba điều kiện)</t>
+          <t>Cho hệ bất phương trình bậc nhất hai ẩn, kiểm tra điểm thuộc miền nghiệm (thay toạ độ vào tất cả các bất phương trình của hệ) - mức Vận dụng, ngoài YCCĐ</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>Pha chế (VDC): số điểm thưởng cao nhất.</t>
+          <t>Cho hệ $2$ hoặc $3$ bất phương trình bậc nhất hai ẩn và $5$ điểm: có bao nhiêu điểm thuộc miền nghiệm của hệ. Số điểm thuộc chọn trước trong $\{1; 2; 3; 4\}$.</t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 1: pha che nuoc); boi_canh pha_che; so lieu ngau nhien cung cau truc</t>
-        </is>
-      </c>
-      <c r="M23" s="3" t="inlineStr">
-        <is>
-          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF; Cùng chữ "Dang" với các chữ B/C (MC/SA) của VD028: cùng dạng nhưng nhiều chữ (khác bối cảnh hoặc khác mức); muc_do_dang = VDC</t>
-        </is>
-      </c>
-      <c r="N23" s="2" t="inlineStr"/>
+          <t>LUYEN TAP THEM - MUC VAN DUNG CAO HON YCCD TH027 CUA BO; CLAUDE THEM 15/10/2026 - co Lan duyet ke hoach ID (diem thuoc mien nghiem cua he; co Lan: he bat phuong</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>Mới 15/10/2026 (dạng điểm thuộc miền nghiệm, ID cô Lan đặt); Luyện tập thêm (ngoài YCCĐ)</t>
+        </is>
+      </c>
+      <c r="N23" s="2" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>B4</t>
+          <t>B3</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>028</t>
+          <t>023</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>VD</t>
+          <t>NB</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1716,68 +1724,56 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_VD028_SA_C</t>
+          <t>L10_C2_B3_NB023_SA_B</t>
         </is>
       </c>
       <c r="G24" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>VDC</t>
-        </is>
-      </c>
-      <c r="I24" s="2" t="inlineStr">
-        <is>
-          <t>pha_che</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="H24" s="2" t="n"/>
+      <c r="I24" s="2" t="n"/>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>Bài toán thực tiễn pha chế nước giải khát: lập bất phương trình, hệ bất phương trình và tìm phương án có điểm thưởng cao nhất (ba điều kiện)</t>
+          <t>Cho bất phương trình ax + by ≤ c (hoặc ≥, &lt;, &gt;) và một nghiệm nguyên M thuộc miền nghiệm: tính giá trị biểu thức F(x; y) = ax + by tại M</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>Pha chế (VDC): số điểm thưởng cao nhất.</t>
+          <t>Trả lời ngắn: tính giá trị $F\left(x; y\right) = ax + by$ (đúng DẠNG này, không có hằng số) tại một nghiệm nguyên $M$ của bất phương trình $ax + by \;\square\; c$ (cùng $a$, $b$ với vế trái).</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 1: pha che nuoc); boi_canh pha_che; so lieu ngau nhien cung cau truc</t>
-        </is>
-      </c>
-      <c r="M24" s="3" t="inlineStr">
-        <is>
-          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF; Cùng chữ "Dang" với các chữ B/C (MC/SA) của VD028: cùng dạng nhưng nhiều chữ (khác bối cảnh hoặc khác mức); muc_do_dang = VDC</t>
-        </is>
-      </c>
-      <c r="N24" s="2" t="inlineStr"/>
+          <t>CLAUDE THEM 29/09/2026 - co Lan kiem tra lai ID va mo ta; 12/10/2026 co Lan: F chi co dang ax + by, M phai thuoc mien nghiem (chon ngau nhien nghiem nguyen); 15</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="n"/>
+      <c r="N24" s="2" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>B4</t>
+          <t>B3</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>028</t>
+          <t>023</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>VD</t>
+          <t>NB</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>TL</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -1787,108 +1783,108 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_VD028_TL_B</t>
+          <t>L10_C2_B3_NB023_MC_B</t>
         </is>
       </c>
       <c r="G25" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H25" s="2" t="inlineStr"/>
-      <c r="I25" s="2" t="inlineStr">
+      <c r="H25" s="2" t="n"/>
+      <c r="I25" s="2" t="n"/>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>Cho bất phương trình ax + by ≤ c (hoặc ≥, &lt;, &gt;) và một nghiệm nguyên M thuộc miền nghiệm: tính giá trị biểu thức F(x; y) = ax + by tại M</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Trắc nghiệm cùng dạng với NB023_SA_B_01: tính $F\left(x; y\right) = ax + by$ tại một nghiệm nguyên $M$.</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>CLAUDE THEM 15/10/2026 - ban trac nghiem cua NB023_SA_B (cung Dang): tinh F = ax + by tai nghiem nguyen M; co Lan duyet lai</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="n"/>
+      <c r="N25" s="2" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>025</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>MC</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>L10_C2_B3_NB025_MC_B</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H26" s="2" t="n"/>
+      <c r="I26" s="2" t="inlineStr">
         <is>
           <t>pha_che</t>
         </is>
       </c>
-      <c r="J25" s="2" t="inlineStr">
+      <c r="J26" s="2" t="inlineStr">
         <is>
           <t>Bài toán thực tiễn pha chế nước giải khát: lập bất phương trình, hệ bất phương trình và tìm phương án có điểm thưởng cao nhất (ba điều kiện)</t>
         </is>
       </c>
-      <c r="K25" s="2" t="inlineStr">
-        <is>
-          <t>Tự luận (2 ý) - pha chế: a) lập hệ bất phương trình (VD); b) phương án có điểm thưởng cao nhất (VDC).</t>
-        </is>
-      </c>
-      <c r="L25" s="2" t="inlineStr">
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Pha chế: bất phương trình về lượng ĐƯỜNG.</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
         <is>
           <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 1: pha che nuoc); boi_canh pha_che; so lieu ngau nhien cung cau truc</t>
         </is>
       </c>
-      <c r="M25" s="3" t="inlineStr">
-        <is>
-          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF</t>
-        </is>
-      </c>
-      <c r="N25" s="2" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr"/>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>(cả chương)</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr"/>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>TF</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>L10_C2_TF_C</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H26" s="2" t="inlineStr"/>
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t>pha_che</t>
-        </is>
-      </c>
-      <c r="J26" s="2" t="inlineStr">
-        <is>
-          <t>Bài toán thực tiễn pha chế nước giải khát: lập bất phương trình, hệ bất phương trình và tìm phương án có điểm thưởng cao nhất (ba điều kiện)</t>
-        </is>
-      </c>
-      <c r="K26" s="2" t="inlineStr">
-        <is>
-          <t>Đúng/Sai theo chương - tình huống pha chế nước (boi_canh pha_che); ý a NB, b TH, c VD, d VDC.</t>
-        </is>
-      </c>
-      <c r="L26" s="2" t="inlineStr">
-        <is>
-          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 1: pha che nuoc); boi_canh pha_che; so lieu ngau nhien cung cau truc</t>
-        </is>
-      </c>
-      <c r="M26" s="3" t="inlineStr">
-        <is>
-          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, 028</t>
-        </is>
-      </c>
-      <c r="N26" s="2" t="inlineStr"/>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>Toán thực tế ở mức NB (quy tắc: thực tế không có NB/TH trừ Đ/S rất dễ) - cần nâng VD/VDC hoặc giữ nếu cô duyệt; Bối cảnh dùng chung với YCCĐ/TF khác: 028, TF</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>B4</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>025</t>
+          <t>028</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>NB</t>
+          <t>VD</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1898,44 +1894,44 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B3_NB025_MC_C</t>
+          <t>L10_C2_B4_VD028_MC_B</t>
         </is>
       </c>
       <c r="G27" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H27" s="2" t="inlineStr"/>
+      <c r="H27" s="2" t="n"/>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>thuc_an_gia_suc</t>
+          <t>pha_che</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>Bài toán thực tiễn thức ăn gia súc: lập bất phương trình, hệ bất phương trình và tìm phương án trộn có chi phí thấp nhất (ba điều kiện dinh dưỡng)</t>
+          <t>Bài toán thực tiễn pha chế nước giải khát: lập bất phương trình, hệ bất phương trình và tìm phương án có điểm thưởng cao nhất (ba điều kiện)</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>Tình huống 2: bất phương trình của điều kiện thứ 1.</t>
+          <t>Pha chế: chọn hệ bất phương trình mô tả đúng các điều kiện.</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 2); boi_canh thuc_an_gia_suc; so lieu ngau nhien cung cau truc</t>
-        </is>
-      </c>
-      <c r="M27" s="3" t="inlineStr">
-        <is>
-          <t>Toán thực tế ở mức NB (quy tắc: thực tế không có NB/TH trừ Đ/S rất dễ) - cần nâng VD/VDC hoặc giữ nếu cô duyệt; Bối cảnh dùng chung với YCCĐ/TF khác: 028, TF</t>
-        </is>
-      </c>
-      <c r="N27" s="2" t="inlineStr"/>
+          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 1: pha che nuoc); boi_canh pha_che; so lieu ngau nhien cung cau truc</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF; Cùng chữ "Dang" với các chữ B/C (MC/SA) của VD028: cùng dạng nhưng nhiều chữ (khác bối cảnh hoặc khác mức)</t>
+        </is>
+      </c>
+      <c r="N27" s="2" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1955,49 +1951,49 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>MC</t>
+          <t>SA</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_VD028_MC_D</t>
+          <t>L10_C2_B4_VD028_SA_B</t>
         </is>
       </c>
       <c r="G28" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H28" s="2" t="inlineStr"/>
+      <c r="H28" s="2" t="n"/>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>thuc_an_gia_suc</t>
+          <t>pha_che</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>Bài toán thực tiễn thức ăn gia súc: lập bất phương trình, hệ bất phương trình và tìm phương án trộn có chi phí thấp nhất (ba điều kiện dinh dưỡng)</t>
+          <t>Bài toán thực tiễn pha chế nước giải khát: lập bất phương trình, hệ bất phương trình và tìm phương án có điểm thưởng cao nhất (ba điều kiện)</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>Tình huống 2 (VD): chọn hệ bất phương trình.</t>
+          <t>Pha chế (VD): số đỉnh của miền nghiệm.</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 2); boi_canh thuc_an_gia_suc; so lieu ngau nhien cung cau truc</t>
-        </is>
-      </c>
-      <c r="M28" s="3" t="inlineStr">
-        <is>
-          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF; Cùng chữ "Dang" với các chữ D/E (MC/SA) của VD028: cùng dạng nhưng nhiều chữ (khác bối cảnh hoặc khác mức)</t>
-        </is>
-      </c>
-      <c r="N28" s="2" t="inlineStr"/>
+          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 1: pha che nuoc); boi_canh pha_che; so lieu ngau nhien cung cau truc</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF; Cùng chữ "Dang" với các chữ B/C (MC/SA) của VD028: cùng dạng nhưng nhiều chữ (khác bối cảnh hoặc khác mức)</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2017,49 +2013,53 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>SA</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_VD028_SA_D</t>
+          <t>L10_C2_B4_VD028_MC_C</t>
         </is>
       </c>
       <c r="G29" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H29" s="2" t="inlineStr"/>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>VDC</t>
+        </is>
+      </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>thuc_an_gia_suc</t>
+          <t>pha_che</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>Bài toán thực tiễn thức ăn gia súc: lập bất phương trình, hệ bất phương trình và tìm phương án trộn có chi phí thấp nhất (ba điều kiện dinh dưỡng)</t>
+          <t>Bài toán thực tiễn pha chế nước giải khát: lập bất phương trình, hệ bất phương trình và tìm phương án có điểm thưởng cao nhất (ba điều kiện)</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>Tình huống 2 (VD): số đỉnh của miền nghiệm.</t>
+          <t>Pha chế (VDC): số điểm thưởng cao nhất.</t>
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 2); boi_canh thuc_an_gia_suc; so lieu ngau nhien cung cau truc</t>
-        </is>
-      </c>
-      <c r="M29" s="3" t="inlineStr">
-        <is>
-          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF; Cùng chữ "Dang" với các chữ D/E (MC/SA) của VD028: cùng dạng nhưng nhiều chữ (khác bối cảnh hoặc khác mức)</t>
-        </is>
-      </c>
-      <c r="N29" s="2" t="inlineStr"/>
+          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 1: pha che nuoc); boi_canh pha_che; so lieu ngau nhien cung cau truc</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF; Cùng chữ "Dang" với các chữ B/C (MC/SA) của VD028: cùng dạng nhưng nhiều chữ (khác bối cảnh hoặc khác mức); muc_do_dang = VDC</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2079,17 +2079,17 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>MC</t>
+          <t>SA</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_VD028_MC_E</t>
+          <t>L10_C2_B4_VD028_SA_C</t>
         </is>
       </c>
       <c r="G30" s="2" t="n">
@@ -2102,30 +2102,30 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>thuc_an_gia_suc</t>
+          <t>pha_che</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>Bài toán thực tiễn thức ăn gia súc: lập bất phương trình, hệ bất phương trình và tìm phương án trộn có chi phí thấp nhất (ba điều kiện dinh dưỡng)</t>
+          <t>Bài toán thực tiễn pha chế nước giải khát: lập bất phương trình, hệ bất phương trình và tìm phương án có điểm thưởng cao nhất (ba điều kiện)</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>Tình huống 2 (VDC): giá trị tối ưu.</t>
+          <t>Pha chế (VDC): số điểm thưởng cao nhất.</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 2); boi_canh thuc_an_gia_suc; so lieu ngau nhien cung cau truc</t>
-        </is>
-      </c>
-      <c r="M30" s="3" t="inlineStr">
-        <is>
-          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF; Cùng chữ "Dang" với các chữ D/E (MC/SA) của VD028: cùng dạng nhưng nhiều chữ (khác bối cảnh hoặc khác mức); muc_do_dang = VDC</t>
-        </is>
-      </c>
-      <c r="N30" s="2" t="inlineStr"/>
+          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 1: pha che nuoc); boi_canh pha_che; so lieu ngau nhien cung cau truc</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF; Cùng chữ "Dang" với các chữ B/C (MC/SA) của VD028: cùng dạng nhưng nhiều chữ (khác bối cảnh hoặc khác mức); muc_do_dang = VDC</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2145,73 +2145,61 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>SA</t>
+          <t>TL</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_VD028_SA_E</t>
+          <t>L10_C2_B4_VD028_TL_B</t>
         </is>
       </c>
       <c r="G31" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="H31" s="2" t="inlineStr">
-        <is>
-          <t>VDC</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="H31" s="2" t="n"/>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>thuc_an_gia_suc</t>
+          <t>pha_che</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>Bài toán thực tiễn thức ăn gia súc: lập bất phương trình, hệ bất phương trình và tìm phương án trộn có chi phí thấp nhất (ba điều kiện dinh dưỡng)</t>
+          <t>Bài toán thực tiễn pha chế nước giải khát: lập bất phương trình, hệ bất phương trình và tìm phương án có điểm thưởng cao nhất (ba điều kiện)</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>Tình huống 2 (VDC): giá trị tối ưu.</t>
+          <t>Tự luận (2 ý) - pha chế: a) lập hệ bất phương trình (VD); b) phương án có điểm thưởng cao nhất (VDC).</t>
         </is>
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 2); boi_canh thuc_an_gia_suc; so lieu ngau nhien cung cau truc</t>
-        </is>
-      </c>
-      <c r="M31" s="3" t="inlineStr">
-        <is>
-          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF; Cùng chữ "Dang" với các chữ D/E (MC/SA) của VD028: cùng dạng nhưng nhiều chữ (khác bối cảnh hoặc khác mức); muc_do_dang = VDC</t>
-        </is>
-      </c>
-      <c r="N31" s="2" t="inlineStr"/>
+          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 1: pha che nuoc); boi_canh pha_che; so lieu ngau nhien cung cau truc</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>B4</t>
-        </is>
-      </c>
+      <c r="A32" s="2" t="n"/>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>028</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>VD</t>
-        </is>
-      </c>
+          <t>(cả chương)</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="n"/>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>TL</t>
+          <t>TF</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -2221,108 +2209,116 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_VD028_TL_C</t>
+          <t>L10_C2_TF_C</t>
         </is>
       </c>
       <c r="G32" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H32" s="2" t="inlineStr"/>
+      <c r="H32" s="2" t="n"/>
       <c r="I32" s="2" t="inlineStr">
         <is>
+          <t>pha_che</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>Bài toán thực tiễn pha chế nước giải khát: lập bất phương trình, hệ bất phương trình và tìm phương án có điểm thưởng cao nhất (ba điều kiện)</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>Đúng/Sai theo chương - tình huống pha chế nước (boi_canh pha_che); ý a NB, b TH, c VD, d VDC.</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 1: pha che nuoc); boi_canh pha_che; so lieu ngau nhien cung cau truc</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, 028</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>025</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>MC</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>L10_C2_B3_NB025_MC_C</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H33" s="2" t="n"/>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
           <t>thuc_an_gia_suc</t>
         </is>
       </c>
-      <c r="J32" s="2" t="inlineStr">
+      <c r="J33" s="2" t="inlineStr">
         <is>
           <t>Bài toán thực tiễn thức ăn gia súc: lập bất phương trình, hệ bất phương trình và tìm phương án trộn có chi phí thấp nhất (ba điều kiện dinh dưỡng)</t>
         </is>
       </c>
-      <c r="K32" s="2" t="inlineStr">
-        <is>
-          <t>Tình huống 2: tự luận 2 ý (a lập hệ, b tối ưu).</t>
-        </is>
-      </c>
-      <c r="L32" s="2" t="inlineStr">
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>Tình huống 2: bất phương trình của điều kiện thứ 1.</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
         <is>
           <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 2); boi_canh thuc_an_gia_suc; so lieu ngau nhien cung cau truc</t>
         </is>
       </c>
-      <c r="M32" s="3" t="inlineStr">
-        <is>
-          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF</t>
-        </is>
-      </c>
-      <c r="N32" s="2" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr"/>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>(cả chương)</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr"/>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>TF</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>L10_C2_TF_D</t>
-        </is>
-      </c>
-      <c r="G33" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H33" s="2" t="inlineStr"/>
-      <c r="I33" s="2" t="inlineStr">
-        <is>
-          <t>thuc_an_gia_suc</t>
-        </is>
-      </c>
-      <c r="J33" s="2" t="inlineStr">
-        <is>
-          <t>Bài toán thực tiễn thức ăn gia súc: lập bất phương trình, hệ bất phương trình và tìm phương án trộn có chi phí thấp nhất (ba điều kiện dinh dưỡng)</t>
-        </is>
-      </c>
-      <c r="K33" s="2" t="inlineStr">
-        <is>
-          <t>Tình huống 2: đúng/sai theo chương, bốn ý.</t>
-        </is>
-      </c>
-      <c r="L33" s="2" t="inlineStr">
-        <is>
-          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 2); boi_canh thuc_an_gia_suc; so lieu ngau nhien cung cau truc</t>
-        </is>
-      </c>
-      <c r="M33" s="3" t="inlineStr">
-        <is>
-          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, 028</t>
-        </is>
-      </c>
-      <c r="N33" s="2" t="inlineStr"/>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>Toán thực tế ở mức NB (quy tắc: thực tế không có NB/TH trừ Đ/S rất dễ) - cần nâng VD/VDC hoặc giữ nếu cô duyệt; Bối cảnh dùng chung với YCCĐ/TF khác: 028, TF</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>B4</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>025</t>
+          <t>028</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>NB</t>
+          <t>VD</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -2337,39 +2333,39 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B3_NB025_MC_D</t>
+          <t>L10_C2_B4_VD028_MC_D</t>
         </is>
       </c>
       <c r="G34" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="H34" s="2" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="H34" s="2" t="n"/>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>phan_xuong_hai_may</t>
+          <t>thuc_an_gia_suc</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>Bài toán thực tiễn phân xưởng hai máy sản xuất hai loại sản phẩm: lập bất phương trình, hệ bất phương trình và tìm phương án có lãi lớn nhất (hai máy)</t>
+          <t>Bài toán thực tiễn thức ăn gia súc: lập bất phương trình, hệ bất phương trình và tìm phương án trộn có chi phí thấp nhất (ba điều kiện dinh dưỡng)</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>Tình huống 3: bất phương trình của điều kiện thứ 1.</t>
+          <t>Tình huống 2 (VD): chọn hệ bất phương trình.</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 3); boi_canh phan_xuong_hai_may; so lieu ngau nhien cung cau truc</t>
-        </is>
-      </c>
-      <c r="M34" s="3" t="inlineStr">
-        <is>
-          <t>Toán thực tế ở mức NB (quy tắc: thực tế không có NB/TH trừ Đ/S rất dễ) - cần nâng VD/VDC hoặc giữ nếu cô duyệt; Bối cảnh dùng chung với YCCĐ/TF khác: 028, TF</t>
-        </is>
-      </c>
-      <c r="N34" s="2" t="inlineStr"/>
+          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 2); boi_canh thuc_an_gia_suc; so lieu ngau nhien cung cau truc</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF; Cùng chữ "Dang" với các chữ D/E (MC/SA) của VD028: cùng dạng nhưng nhiều chữ (khác bối cảnh hoặc khác mức)</t>
+        </is>
+      </c>
+      <c r="N34" s="2" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2389,49 +2385,49 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>MC</t>
+          <t>SA</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_VD028_MC_F</t>
+          <t>L10_C2_B4_VD028_SA_D</t>
         </is>
       </c>
       <c r="G35" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H35" s="2" t="inlineStr"/>
+      <c r="H35" s="2" t="n"/>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>phan_xuong_hai_may</t>
+          <t>thuc_an_gia_suc</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>Bài toán thực tiễn phân xưởng hai máy sản xuất hai loại sản phẩm: lập bất phương trình, hệ bất phương trình và tìm phương án có lãi lớn nhất (hai máy)</t>
+          <t>Bài toán thực tiễn thức ăn gia súc: lập bất phương trình, hệ bất phương trình và tìm phương án trộn có chi phí thấp nhất (ba điều kiện dinh dưỡng)</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>Tình huống 3 (VD): chọn hệ bất phương trình.</t>
+          <t>Tình huống 2 (VD): số đỉnh của miền nghiệm.</t>
         </is>
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 3); boi_canh phan_xuong_hai_may; so lieu ngau nhien cung cau truc</t>
-        </is>
-      </c>
-      <c r="M35" s="3" t="inlineStr">
-        <is>
-          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF; Cùng chữ "Dang" với các chữ F/G (MC/SA) của VD028: cùng dạng nhưng nhiều chữ (khác bối cảnh hoặc khác mức)</t>
-        </is>
-      </c>
-      <c r="N35" s="2" t="inlineStr"/>
+          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 2); boi_canh thuc_an_gia_suc; so lieu ngau nhien cung cau truc</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF; Cùng chữ "Dang" với các chữ D/E (MC/SA) của VD028: cùng dạng nhưng nhiều chữ (khác bối cảnh hoặc khác mức)</t>
+        </is>
+      </c>
+      <c r="N35" s="2" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2451,49 +2447,53 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>SA</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_VD028_SA_F</t>
+          <t>L10_C2_B4_VD028_MC_E</t>
         </is>
       </c>
       <c r="G36" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H36" s="2" t="inlineStr"/>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>VDC</t>
+        </is>
+      </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>phan_xuong_hai_may</t>
+          <t>thuc_an_gia_suc</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>Bài toán thực tiễn phân xưởng hai máy sản xuất hai loại sản phẩm: lập bất phương trình, hệ bất phương trình và tìm phương án có lãi lớn nhất (hai máy)</t>
+          <t>Bài toán thực tiễn thức ăn gia súc: lập bất phương trình, hệ bất phương trình và tìm phương án trộn có chi phí thấp nhất (ba điều kiện dinh dưỡng)</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>Tình huống 3 (VD): số đỉnh của miền nghiệm.</t>
+          <t>Tình huống 2 (VDC): giá trị tối ưu.</t>
         </is>
       </c>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 3); boi_canh phan_xuong_hai_may; so lieu ngau nhien cung cau truc</t>
-        </is>
-      </c>
-      <c r="M36" s="3" t="inlineStr">
-        <is>
-          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF; Cùng chữ "Dang" với các chữ F/G (MC/SA) của VD028: cùng dạng nhưng nhiều chữ (khác bối cảnh hoặc khác mức)</t>
-        </is>
-      </c>
-      <c r="N36" s="2" t="inlineStr"/>
+          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 2); boi_canh thuc_an_gia_suc; so lieu ngau nhien cung cau truc</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF; Cùng chữ "Dang" với các chữ D/E (MC/SA) của VD028: cùng dạng nhưng nhiều chữ (khác bối cảnh hoặc khác mức); muc_do_dang = VDC</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2513,17 +2513,17 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>MC</t>
+          <t>SA</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>E</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_VD028_MC_G</t>
+          <t>L10_C2_B4_VD028_SA_E</t>
         </is>
       </c>
       <c r="G37" s="2" t="n">
@@ -2536,30 +2536,30 @@
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>phan_xuong_hai_may</t>
+          <t>thuc_an_gia_suc</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>Bài toán thực tiễn phân xưởng hai máy sản xuất hai loại sản phẩm: lập bất phương trình, hệ bất phương trình và tìm phương án có lãi lớn nhất (hai máy)</t>
+          <t>Bài toán thực tiễn thức ăn gia súc: lập bất phương trình, hệ bất phương trình và tìm phương án trộn có chi phí thấp nhất (ba điều kiện dinh dưỡng)</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>Tình huống 3 (VDC): giá trị tối ưu.</t>
+          <t>Tình huống 2 (VDC): giá trị tối ưu.</t>
         </is>
       </c>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 3); boi_canh phan_xuong_hai_may; so lieu ngau nhien cung cau truc</t>
-        </is>
-      </c>
-      <c r="M37" s="3" t="inlineStr">
-        <is>
-          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF; Cùng chữ "Dang" với các chữ F/G (MC/SA) của VD028: cùng dạng nhưng nhiều chữ (khác bối cảnh hoặc khác mức); muc_do_dang = VDC</t>
-        </is>
-      </c>
-      <c r="N37" s="2" t="inlineStr"/>
+          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 2); boi_canh thuc_an_gia_suc; so lieu ngau nhien cung cau truc</t>
+        </is>
+      </c>
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF; Cùng chữ "Dang" với các chữ D/E (MC/SA) của VD028: cùng dạng nhưng nhiều chữ (khác bối cảnh hoặc khác mức); muc_do_dang = VDC</t>
+        </is>
+      </c>
+      <c r="N37" s="2" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2579,73 +2579,61 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>SA</t>
+          <t>TL</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_VD028_SA_G</t>
+          <t>L10_C2_B4_VD028_TL_C</t>
         </is>
       </c>
       <c r="G38" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="H38" s="2" t="inlineStr">
-        <is>
-          <t>VDC</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="H38" s="2" t="n"/>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>phan_xuong_hai_may</t>
+          <t>thuc_an_gia_suc</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>Bài toán thực tiễn phân xưởng hai máy sản xuất hai loại sản phẩm: lập bất phương trình, hệ bất phương trình và tìm phương án có lãi lớn nhất (hai máy)</t>
+          <t>Bài toán thực tiễn thức ăn gia súc: lập bất phương trình, hệ bất phương trình và tìm phương án trộn có chi phí thấp nhất (ba điều kiện dinh dưỡng)</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>Tình huống 3 (VDC): giá trị tối ưu.</t>
+          <t>Tình huống 2: tự luận 2 ý (a lập hệ, b tối ưu).</t>
         </is>
       </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 3); boi_canh phan_xuong_hai_may; so lieu ngau nhien cung cau truc</t>
-        </is>
-      </c>
-      <c r="M38" s="3" t="inlineStr">
-        <is>
-          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF; Cùng chữ "Dang" với các chữ F/G (MC/SA) của VD028: cùng dạng nhưng nhiều chữ (khác bối cảnh hoặc khác mức); muc_do_dang = VDC</t>
-        </is>
-      </c>
-      <c r="N38" s="2" t="inlineStr"/>
+          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 2); boi_canh thuc_an_gia_suc; so lieu ngau nhien cung cau truc</t>
+        </is>
+      </c>
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF</t>
+        </is>
+      </c>
+      <c r="N38" s="2" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>B4</t>
-        </is>
-      </c>
+      <c r="A39" s="2" t="n"/>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>028</t>
-        </is>
-      </c>
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t>VD</t>
-        </is>
-      </c>
+          <t>(cả chương)</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="n"/>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>TL</t>
+          <t>TF</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -2655,108 +2643,116 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_VD028_TL_D</t>
+          <t>L10_C2_TF_D</t>
         </is>
       </c>
       <c r="G39" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H39" s="2" t="inlineStr"/>
+      <c r="H39" s="2" t="n"/>
       <c r="I39" s="2" t="inlineStr">
         <is>
+          <t>thuc_an_gia_suc</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>Bài toán thực tiễn thức ăn gia súc: lập bất phương trình, hệ bất phương trình và tìm phương án trộn có chi phí thấp nhất (ba điều kiện dinh dưỡng)</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>Tình huống 2: đúng/sai theo chương, bốn ý.</t>
+        </is>
+      </c>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 2); boi_canh thuc_an_gia_suc; so lieu ngau nhien cung cau truc</t>
+        </is>
+      </c>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, 028</t>
+        </is>
+      </c>
+      <c r="N39" s="2" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>025</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>MC</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>L10_C2_B3_NB025_MC_D</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H40" s="2" t="n"/>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
           <t>phan_xuong_hai_may</t>
         </is>
       </c>
-      <c r="J39" s="2" t="inlineStr">
+      <c r="J40" s="2" t="inlineStr">
         <is>
           <t>Bài toán thực tiễn phân xưởng hai máy sản xuất hai loại sản phẩm: lập bất phương trình, hệ bất phương trình và tìm phương án có lãi lớn nhất (hai máy)</t>
         </is>
       </c>
-      <c r="K39" s="2" t="inlineStr">
-        <is>
-          <t>Tình huống 3: tự luận 2 ý (a lập hệ, b tối ưu).</t>
-        </is>
-      </c>
-      <c r="L39" s="2" t="inlineStr">
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>Tình huống 3: bất phương trình của điều kiện thứ 1.</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr">
         <is>
           <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 3); boi_canh phan_xuong_hai_may; so lieu ngau nhien cung cau truc</t>
         </is>
       </c>
-      <c r="M39" s="3" t="inlineStr">
-        <is>
-          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF</t>
-        </is>
-      </c>
-      <c r="N39" s="2" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr"/>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>(cả chương)</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="inlineStr"/>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>TF</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="F40" s="2" t="inlineStr">
-        <is>
-          <t>L10_C2_TF_E</t>
-        </is>
-      </c>
-      <c r="G40" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H40" s="2" t="inlineStr"/>
-      <c r="I40" s="2" t="inlineStr">
-        <is>
-          <t>phan_xuong_hai_may</t>
-        </is>
-      </c>
-      <c r="J40" s="2" t="inlineStr">
-        <is>
-          <t>Bài toán thực tiễn phân xưởng hai máy sản xuất hai loại sản phẩm: lập bất phương trình, hệ bất phương trình và tìm phương án có lãi lớn nhất (hai máy)</t>
-        </is>
-      </c>
-      <c r="K40" s="2" t="inlineStr">
-        <is>
-          <t>Tình huống 3: đúng/sai theo chương, bốn ý.</t>
-        </is>
-      </c>
-      <c r="L40" s="2" t="inlineStr">
-        <is>
-          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 3); boi_canh phan_xuong_hai_may; so lieu ngau nhien cung cau truc</t>
-        </is>
-      </c>
-      <c r="M40" s="3" t="inlineStr">
-        <is>
-          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, 028</t>
-        </is>
-      </c>
-      <c r="N40" s="2" t="inlineStr"/>
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>Toán thực tế ở mức NB (quy tắc: thực tế không có NB/TH trừ Đ/S rất dễ) - cần nâng VD/VDC hoặc giữ nếu cô duyệt; Bối cảnh dùng chung với YCCĐ/TF khác: 028, TF</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>B4</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>025</t>
+          <t>028</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>NB</t>
+          <t>VD</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -2766,44 +2762,44 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B3_NB025_MC_E</t>
+          <t>L10_C2_B4_VD028_MC_F</t>
         </is>
       </c>
       <c r="G41" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H41" s="2" t="inlineStr"/>
+      <c r="H41" s="2" t="n"/>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>do_uong_an_kieng</t>
+          <t>phan_xuong_hai_may</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>Bài toán thực tiễn đồ uống ăn kiêng: lập bất phương trình, hệ bất phương trình và tìm phương án có chi phí thấp nhất (calo và hai loại vitamin)</t>
+          <t>Bài toán thực tiễn phân xưởng hai máy sản xuất hai loại sản phẩm: lập bất phương trình, hệ bất phương trình và tìm phương án có lãi lớn nhất (hai máy)</t>
         </is>
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>Tình huống 4: bất phương trình của điều kiện thứ 1.</t>
+          <t>Tình huống 3 (VD): chọn hệ bất phương trình.</t>
         </is>
       </c>
       <c r="L41" s="2" t="inlineStr">
         <is>
-          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 4); boi_canh do_uong_an_kieng; so lieu ngau nhien cung cau truc</t>
-        </is>
-      </c>
-      <c r="M41" s="3" t="inlineStr">
-        <is>
-          <t>Toán thực tế ở mức NB (quy tắc: thực tế không có NB/TH trừ Đ/S rất dễ) - cần nâng VD/VDC hoặc giữ nếu cô duyệt; Bối cảnh dùng chung với YCCĐ/TF khác: 028, TF</t>
-        </is>
-      </c>
-      <c r="N41" s="2" t="inlineStr"/>
+          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 3); boi_canh phan_xuong_hai_may; so lieu ngau nhien cung cau truc</t>
+        </is>
+      </c>
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF; Cùng chữ "Dang" với các chữ F/G (MC/SA) của VD028: cùng dạng nhưng nhiều chữ (khác bối cảnh hoặc khác mức)</t>
+        </is>
+      </c>
+      <c r="N41" s="2" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2823,49 +2819,49 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>MC</t>
+          <t>SA</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_VD028_MC_H</t>
+          <t>L10_C2_B4_VD028_SA_F</t>
         </is>
       </c>
       <c r="G42" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H42" s="2" t="inlineStr"/>
+      <c r="H42" s="2" t="n"/>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>do_uong_an_kieng</t>
+          <t>phan_xuong_hai_may</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>Bài toán thực tiễn đồ uống ăn kiêng: lập bất phương trình, hệ bất phương trình và tìm phương án có chi phí thấp nhất (calo và hai loại vitamin)</t>
+          <t>Bài toán thực tiễn phân xưởng hai máy sản xuất hai loại sản phẩm: lập bất phương trình, hệ bất phương trình và tìm phương án có lãi lớn nhất (hai máy)</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>Tình huống 4 (VD): chọn hệ bất phương trình.</t>
+          <t>Tình huống 3 (VD): số đỉnh của miền nghiệm.</t>
         </is>
       </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 4); boi_canh do_uong_an_kieng; so lieu ngau nhien cung cau truc</t>
-        </is>
-      </c>
-      <c r="M42" s="3" t="inlineStr">
-        <is>
-          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF; Cùng chữ "Dang" với các chữ H/I (MC/SA) của VD028: cùng dạng nhưng nhiều chữ (khác bối cảnh hoặc khác mức)</t>
-        </is>
-      </c>
-      <c r="N42" s="2" t="inlineStr"/>
+          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 3); boi_canh phan_xuong_hai_may; so lieu ngau nhien cung cau truc</t>
+        </is>
+      </c>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF; Cùng chữ "Dang" với các chữ F/G (MC/SA) của VD028: cùng dạng nhưng nhiều chữ (khác bối cảnh hoặc khác mức)</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -2885,49 +2881,53 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>SA</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>G</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_VD028_SA_H</t>
+          <t>L10_C2_B4_VD028_MC_G</t>
         </is>
       </c>
       <c r="G43" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H43" s="2" t="inlineStr"/>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>VDC</t>
+        </is>
+      </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>do_uong_an_kieng</t>
+          <t>phan_xuong_hai_may</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>Bài toán thực tiễn đồ uống ăn kiêng: lập bất phương trình, hệ bất phương trình và tìm phương án có chi phí thấp nhất (calo và hai loại vitamin)</t>
+          <t>Bài toán thực tiễn phân xưởng hai máy sản xuất hai loại sản phẩm: lập bất phương trình, hệ bất phương trình và tìm phương án có lãi lớn nhất (hai máy)</t>
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>Tình huống 4 (VD): số đỉnh của miền nghiệm.</t>
+          <t>Tình huống 3 (VDC): giá trị tối ưu.</t>
         </is>
       </c>
       <c r="L43" s="2" t="inlineStr">
         <is>
-          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 4); boi_canh do_uong_an_kieng; so lieu ngau nhien cung cau truc</t>
-        </is>
-      </c>
-      <c r="M43" s="3" t="inlineStr">
-        <is>
-          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF; Cùng chữ "Dang" với các chữ H/I (MC/SA) của VD028: cùng dạng nhưng nhiều chữ (khác bối cảnh hoặc khác mức)</t>
-        </is>
-      </c>
-      <c r="N43" s="2" t="inlineStr"/>
+          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 3); boi_canh phan_xuong_hai_may; so lieu ngau nhien cung cau truc</t>
+        </is>
+      </c>
+      <c r="M43" s="2" t="inlineStr">
+        <is>
+          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF; Cùng chữ "Dang" với các chữ F/G (MC/SA) của VD028: cùng dạng nhưng nhiều chữ (khác bối cảnh hoặc khác mức); muc_do_dang = VDC</t>
+        </is>
+      </c>
+      <c r="N43" s="2" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -2947,17 +2947,17 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>MC</t>
+          <t>SA</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>G</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_VD028_MC_I</t>
+          <t>L10_C2_B4_VD028_SA_G</t>
         </is>
       </c>
       <c r="G44" s="2" t="n">
@@ -2970,30 +2970,30 @@
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>do_uong_an_kieng</t>
+          <t>phan_xuong_hai_may</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>Bài toán thực tiễn đồ uống ăn kiêng: lập bất phương trình, hệ bất phương trình và tìm phương án có chi phí thấp nhất (calo và hai loại vitamin)</t>
+          <t>Bài toán thực tiễn phân xưởng hai máy sản xuất hai loại sản phẩm: lập bất phương trình, hệ bất phương trình và tìm phương án có lãi lớn nhất (hai máy)</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>Tình huống 4 (VDC): giá trị tối ưu.</t>
+          <t>Tình huống 3 (VDC): giá trị tối ưu.</t>
         </is>
       </c>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 4); boi_canh do_uong_an_kieng; so lieu ngau nhien cung cau truc</t>
-        </is>
-      </c>
-      <c r="M44" s="3" t="inlineStr">
-        <is>
-          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF; Cùng chữ "Dang" với các chữ H/I (MC/SA) của VD028: cùng dạng nhưng nhiều chữ (khác bối cảnh hoặc khác mức); muc_do_dang = VDC</t>
-        </is>
-      </c>
-      <c r="N44" s="2" t="inlineStr"/>
+          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 3); boi_canh phan_xuong_hai_may; so lieu ngau nhien cung cau truc</t>
+        </is>
+      </c>
+      <c r="M44" s="2" t="inlineStr">
+        <is>
+          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF; Cùng chữ "Dang" với các chữ F/G (MC/SA) của VD028: cùng dạng nhưng nhiều chữ (khác bối cảnh hoặc khác mức); muc_do_dang = VDC</t>
+        </is>
+      </c>
+      <c r="N44" s="2" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3013,73 +3013,61 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>SA</t>
+          <t>TL</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>D</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_VD028_SA_I</t>
+          <t>L10_C2_B4_VD028_TL_D</t>
         </is>
       </c>
       <c r="G45" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="H45" s="2" t="inlineStr">
-        <is>
-          <t>VDC</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="H45" s="2" t="n"/>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>do_uong_an_kieng</t>
+          <t>phan_xuong_hai_may</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>Bài toán thực tiễn đồ uống ăn kiêng: lập bất phương trình, hệ bất phương trình và tìm phương án có chi phí thấp nhất (calo và hai loại vitamin)</t>
+          <t>Bài toán thực tiễn phân xưởng hai máy sản xuất hai loại sản phẩm: lập bất phương trình, hệ bất phương trình và tìm phương án có lãi lớn nhất (hai máy)</t>
         </is>
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>Tình huống 4 (VDC): giá trị tối ưu.</t>
+          <t>Tình huống 3: tự luận 2 ý (a lập hệ, b tối ưu).</t>
         </is>
       </c>
       <c r="L45" s="2" t="inlineStr">
         <is>
-          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 4); boi_canh do_uong_an_kieng; so lieu ngau nhien cung cau truc</t>
-        </is>
-      </c>
-      <c r="M45" s="3" t="inlineStr">
-        <is>
-          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF; Cùng chữ "Dang" với các chữ H/I (MC/SA) của VD028: cùng dạng nhưng nhiều chữ (khác bối cảnh hoặc khác mức); muc_do_dang = VDC</t>
-        </is>
-      </c>
-      <c r="N45" s="2" t="inlineStr"/>
+          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 3); boi_canh phan_xuong_hai_may; so lieu ngau nhien cung cau truc</t>
+        </is>
+      </c>
+      <c r="M45" s="2" t="inlineStr">
+        <is>
+          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF</t>
+        </is>
+      </c>
+      <c r="N45" s="2" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>B4</t>
-        </is>
-      </c>
+      <c r="A46" s="2" t="n"/>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>028</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>VD</t>
-        </is>
-      </c>
+          <t>(cả chương)</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="n"/>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>TL</t>
+          <t>TF</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -3089,93 +3077,101 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_VD028_TL_E</t>
+          <t>L10_C2_TF_E</t>
         </is>
       </c>
       <c r="G46" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H46" s="2" t="inlineStr"/>
+      <c r="H46" s="2" t="n"/>
       <c r="I46" s="2" t="inlineStr">
         <is>
+          <t>phan_xuong_hai_may</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>Bài toán thực tiễn phân xưởng hai máy sản xuất hai loại sản phẩm: lập bất phương trình, hệ bất phương trình và tìm phương án có lãi lớn nhất (hai máy)</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>Tình huống 3: đúng/sai theo chương, bốn ý.</t>
+        </is>
+      </c>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 3); boi_canh phan_xuong_hai_may; so lieu ngau nhien cung cau truc</t>
+        </is>
+      </c>
+      <c r="M46" s="2" t="inlineStr">
+        <is>
+          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, 028</t>
+        </is>
+      </c>
+      <c r="N46" s="2" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>025</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>NB</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>MC</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>L10_C2_B3_NB025_MC_E</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H47" s="2" t="n"/>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
           <t>do_uong_an_kieng</t>
         </is>
       </c>
-      <c r="J46" s="2" t="inlineStr">
+      <c r="J47" s="2" t="inlineStr">
         <is>
           <t>Bài toán thực tiễn đồ uống ăn kiêng: lập bất phương trình, hệ bất phương trình và tìm phương án có chi phí thấp nhất (calo và hai loại vitamin)</t>
         </is>
       </c>
-      <c r="K46" s="2" t="inlineStr">
-        <is>
-          <t>Tình huống 4: tự luận 2 ý (a lập hệ, b tối ưu).</t>
-        </is>
-      </c>
-      <c r="L46" s="2" t="inlineStr">
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>Tình huống 4: bất phương trình của điều kiện thứ 1.</t>
+        </is>
+      </c>
+      <c r="L47" s="2" t="inlineStr">
         <is>
           <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 4); boi_canh do_uong_an_kieng; so lieu ngau nhien cung cau truc</t>
         </is>
       </c>
-      <c r="M46" s="3" t="inlineStr">
-        <is>
-          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF</t>
-        </is>
-      </c>
-      <c r="N46" s="2" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr"/>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>(cả chương)</t>
-        </is>
-      </c>
-      <c r="C47" s="2" t="inlineStr"/>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>TF</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="F47" s="2" t="inlineStr">
-        <is>
-          <t>L10_C2_TF_F</t>
-        </is>
-      </c>
-      <c r="G47" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H47" s="2" t="inlineStr"/>
-      <c r="I47" s="2" t="inlineStr">
-        <is>
-          <t>do_uong_an_kieng</t>
-        </is>
-      </c>
-      <c r="J47" s="2" t="inlineStr">
-        <is>
-          <t>Bài toán thực tiễn đồ uống ăn kiêng: lập bất phương trình, hệ bất phương trình và tìm phương án có chi phí thấp nhất (calo và hai loại vitamin)</t>
-        </is>
-      </c>
-      <c r="K47" s="2" t="inlineStr">
-        <is>
-          <t>Tình huống 4: đúng/sai theo chương, bốn ý.</t>
-        </is>
-      </c>
-      <c r="L47" s="2" t="inlineStr">
-        <is>
-          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 4); boi_canh do_uong_an_kieng; so lieu ngau nhien cung cau truc</t>
-        </is>
-      </c>
-      <c r="M47" s="3" t="inlineStr">
-        <is>
-          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, 028</t>
-        </is>
-      </c>
-      <c r="N47" s="2" t="inlineStr"/>
+      <c r="M47" s="2" t="inlineStr">
+        <is>
+          <t>Toán thực tế ở mức NB (quy tắc: thực tế không có NB/TH trừ Đ/S rất dễ) - cần nâng VD/VDC hoặc giữ nếu cô duyệt; Bối cảnh dùng chung với YCCĐ/TF khác: 028, TF</t>
+        </is>
+      </c>
+      <c r="N47" s="2" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3200,40 +3196,44 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>H</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_VD028_MC_J</t>
+          <t>L10_C2_B4_VD028_MC_H</t>
         </is>
       </c>
       <c r="G48" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H48" s="2" t="inlineStr"/>
-      <c r="I48" s="2" t="inlineStr"/>
+      <c r="H48" s="2" t="n"/>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>do_uong_an_kieng</t>
+        </is>
+      </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>Diện tích và toạ độ đỉnh của miền nghiệm là tam giác của hệ ba bất phương trình (một bất phương trình song song với trục toạ độ)</t>
+          <t>Bài toán thực tiễn đồ uống ăn kiêng: lập bất phương trình, hệ bất phương trình và tìm phương án có chi phí thấp nhất (calo và hai loại vitamin)</t>
         </is>
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>Diện tích miền nghiệm (tam giác) của hệ ba bất phương trình, một bất phương trình song song Ox hoặc Oy.</t>
+          <t>Tình huống 4 (VD): chọn hệ bất phương trình.</t>
         </is>
       </c>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>LUYEN TAP THEM - khong co trong yeu cau can dat cua Bo (dien tich mien nghiem la tam giac, he 3 bat phuong trinh co 1 bpt song song Ox hoac Oy). CLAUDE THEM 09/</t>
-        </is>
-      </c>
-      <c r="M48" s="3" t="inlineStr">
-        <is>
-          <t>Luyện tập thêm (ngoài YCCĐ)</t>
-        </is>
-      </c>
-      <c r="N48" s="2" t="inlineStr"/>
+          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 4); boi_canh do_uong_an_kieng; so lieu ngau nhien cung cau truc</t>
+        </is>
+      </c>
+      <c r="M48" s="2" t="inlineStr">
+        <is>
+          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF; Cùng chữ "Dang" với các chữ H/I (MC/SA) của VD028: cùng dạng nhưng nhiều chữ (khác bối cảnh hoặc khác mức)</t>
+        </is>
+      </c>
+      <c r="N48" s="2" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3258,40 +3258,44 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>H</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_VD028_SA_J</t>
+          <t>L10_C2_B4_VD028_SA_H</t>
         </is>
       </c>
       <c r="G49" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="H49" s="2" t="inlineStr"/>
-      <c r="I49" s="2" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="H49" s="2" t="n"/>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>do_uong_an_kieng</t>
+        </is>
+      </c>
       <c r="J49" s="2" t="inlineStr">
         <is>
-          <t>Diện tích và toạ độ đỉnh của miền nghiệm là tam giác của hệ ba bất phương trình (một bất phương trình song song với trục toạ độ)</t>
+          <t>Bài toán thực tiễn đồ uống ăn kiêng: lập bất phương trình, hệ bất phương trình và tìm phương án có chi phí thấp nhất (calo và hai loại vitamin)</t>
         </is>
       </c>
       <c r="K49" s="2" t="inlineStr">
         <is>
-          <t>Diện tích miền nghiệm (tam giác).</t>
+          <t>Tình huống 4 (VD): số đỉnh của miền nghiệm.</t>
         </is>
       </c>
       <c r="L49" s="2" t="inlineStr">
         <is>
-          <t>LUYEN TAP THEM - khong co trong yeu cau can dat cua Bo (dien tich mien nghiem la tam giac, he 3 bat phuong trinh co 1 bpt song song Ox hoac Oy). CLAUDE THEM 09/</t>
-        </is>
-      </c>
-      <c r="M49" s="3" t="inlineStr">
-        <is>
-          <t>Luyện tập thêm (ngoài YCCĐ)</t>
-        </is>
-      </c>
-      <c r="N49" s="2" t="inlineStr"/>
+          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 4); boi_canh do_uong_an_kieng; so lieu ngau nhien cung cau truc</t>
+        </is>
+      </c>
+      <c r="M49" s="2" t="inlineStr">
+        <is>
+          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF; Cùng chữ "Dang" với các chữ H/I (MC/SA) của VD028: cùng dạng nhưng nhiều chữ (khác bối cảnh hoặc khác mức)</t>
+        </is>
+      </c>
+      <c r="N49" s="2" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3316,44 +3320,48 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>I</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_VD028_MC_K</t>
+          <t>L10_C2_B4_VD028_MC_I</t>
         </is>
       </c>
       <c r="G50" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
           <t>VDC</t>
         </is>
       </c>
-      <c r="I50" s="2" t="inlineStr"/>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>do_uong_an_kieng</t>
+        </is>
+      </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>Tìm tham số m khi biết diện tích tam giác là miền nghiệm của hệ ba bất phương trình (bất phương trình song song với trục chứa tham số)</t>
+          <t>Bài toán thực tiễn đồ uống ăn kiêng: lập bất phương trình, hệ bất phương trình và tìm phương án có chi phí thấp nhất (calo và hai loại vitamin)</t>
         </is>
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>Có tham số (VDC): biết diện tích tam giác, tìm m.</t>
+          <t>Tình huống 4 (VDC): giá trị tối ưu.</t>
         </is>
       </c>
       <c r="L50" s="2" t="inlineStr">
         <is>
-          <t>LUYEN TAP THEM - khong co trong yeu cau can dat cua Bo (dien tich mien nghiem la tam giac, he 3 bat phuong trinh co 1 bpt song song Ox hoac Oy). CLAUDE THEM 09/</t>
-        </is>
-      </c>
-      <c r="M50" s="3" t="inlineStr">
-        <is>
-          <t>muc_do_dang = VDC; Luyện tập thêm (ngoài YCCĐ)</t>
-        </is>
-      </c>
-      <c r="N50" s="2" t="inlineStr"/>
+          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 4); boi_canh do_uong_an_kieng; so lieu ngau nhien cung cau truc</t>
+        </is>
+      </c>
+      <c r="M50" s="2" t="inlineStr">
+        <is>
+          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF; Cùng chữ "Dang" với các chữ H/I (MC/SA) của VD028: cùng dạng nhưng nhiều chữ (khác bối cảnh hoặc khác mức); muc_do_dang = VDC</t>
+        </is>
+      </c>
+      <c r="N50" s="2" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3378,44 +3386,48 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>I</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_VD028_SA_K</t>
+          <t>L10_C2_B4_VD028_SA_I</t>
         </is>
       </c>
       <c r="G51" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
           <t>VDC</t>
         </is>
       </c>
-      <c r="I51" s="2" t="inlineStr"/>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>do_uong_an_kieng</t>
+        </is>
+      </c>
       <c r="J51" s="2" t="inlineStr">
         <is>
-          <t>Tìm tham số m khi biết diện tích tam giác là miền nghiệm của hệ ba bất phương trình (bất phương trình song song với trục chứa tham số)</t>
+          <t>Bài toán thực tiễn đồ uống ăn kiêng: lập bất phương trình, hệ bất phương trình và tìm phương án có chi phí thấp nhất (calo và hai loại vitamin)</t>
         </is>
       </c>
       <c r="K51" s="2" t="inlineStr">
         <is>
-          <t>Có tham số (VDC): tìm m.</t>
+          <t>Tình huống 4 (VDC): giá trị tối ưu.</t>
         </is>
       </c>
       <c r="L51" s="2" t="inlineStr">
         <is>
-          <t>LUYEN TAP THEM - khong co trong yeu cau can dat cua Bo (dien tich mien nghiem la tam giac, he 3 bat phuong trinh co 1 bpt song song Ox hoac Oy). CLAUDE THEM 09/</t>
-        </is>
-      </c>
-      <c r="M51" s="3" t="inlineStr">
-        <is>
-          <t>muc_do_dang = VDC; Luyện tập thêm (ngoài YCCĐ)</t>
-        </is>
-      </c>
-      <c r="N51" s="2" t="inlineStr"/>
+          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 4); boi_canh do_uong_an_kieng; so lieu ngau nhien cung cau truc</t>
+        </is>
+      </c>
+      <c r="M51" s="2" t="inlineStr">
+        <is>
+          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF; Cùng chữ "Dang" với các chữ H/I (MC/SA) của VD028: cùng dạng nhưng nhiều chữ (khác bối cảnh hoặc khác mức); muc_do_dang = VDC</t>
+        </is>
+      </c>
+      <c r="N51" s="2" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3440,101 +3452,457 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_VD028_TL_F</t>
+          <t>L10_C2_B4_VD028_TL_E</t>
         </is>
       </c>
       <c r="G52" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H52" s="2" t="inlineStr"/>
-      <c r="I52" s="2" t="inlineStr"/>
+      <c r="H52" s="2" t="n"/>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>do_uong_an_kieng</t>
+        </is>
+      </c>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>Diện tích và toạ độ đỉnh của miền nghiệm là tam giác của hệ ba bất phương trình (một bất phương trình song song với trục toạ độ)</t>
+          <t>Bài toán thực tiễn đồ uống ăn kiêng: lập bất phương trình, hệ bất phương trình và tìm phương án có chi phí thấp nhất (calo và hai loại vitamin)</t>
         </is>
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>Tự luận 2 ý: a) toạ độ các đỉnh, b) diện tích tam giác miền nghiệm.</t>
+          <t>Tình huống 4: tự luận 2 ý (a lập hệ, b tối ưu).</t>
         </is>
       </c>
       <c r="L52" s="2" t="inlineStr">
         <is>
-          <t>LUYEN TAP THEM - khong co trong yeu cau can dat cua Bo (dien tich mien nghiem la tam giac, he 3 bat phuong trinh co 1 bpt song song Ox hoac Oy). CLAUDE THEM 09/</t>
-        </is>
-      </c>
-      <c r="M52" s="3" t="inlineStr">
-        <is>
-          <t>Luyện tập thêm (ngoài YCCĐ)</t>
-        </is>
-      </c>
-      <c r="N52" s="2" t="inlineStr"/>
+          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 4); boi_canh do_uong_an_kieng; so lieu ngau nhien cung cau truc</t>
+        </is>
+      </c>
+      <c r="M52" s="2" t="inlineStr">
+        <is>
+          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF</t>
+        </is>
+      </c>
+      <c r="N52" s="2" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="inlineStr">
-        <is>
-          <t>B4</t>
-        </is>
-      </c>
+      <c r="A53" s="2" t="n"/>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>028</t>
-        </is>
-      </c>
-      <c r="C53" s="2" t="inlineStr">
-        <is>
-          <t>VD</t>
-        </is>
-      </c>
+          <t>(cả chương)</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="n"/>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>TL</t>
+          <t>TF</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_VD028_TL_G</t>
+          <t>L10_C2_TF_F</t>
         </is>
       </c>
       <c r="G53" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H53" s="2" t="inlineStr"/>
-      <c r="I53" s="2" t="inlineStr"/>
+      <c r="H53" s="2" t="n"/>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>do_uong_an_kieng</t>
+        </is>
+      </c>
       <c r="J53" s="2" t="inlineStr">
         <is>
+          <t>Bài toán thực tiễn đồ uống ăn kiêng: lập bất phương trình, hệ bất phương trình và tìm phương án có chi phí thấp nhất (calo và hai loại vitamin)</t>
+        </is>
+      </c>
+      <c r="K53" s="2" t="inlineStr">
+        <is>
+          <t>Tình huống 4: đúng/sai theo chương, bốn ý.</t>
+        </is>
+      </c>
+      <c r="L53" s="2" t="inlineStr">
+        <is>
+          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 4); boi_canh do_uong_an_kieng; so lieu ngau nhien cung cau truc</t>
+        </is>
+      </c>
+      <c r="M53" s="2" t="inlineStr">
+        <is>
+          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, 028</t>
+        </is>
+      </c>
+      <c r="N53" s="2" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>B4</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>028</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>VD</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>MC</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>L10_C2_B4_VD028_MC_J</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H54" s="2" t="n"/>
+      <c r="I54" s="2" t="n"/>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>Diện tích và toạ độ đỉnh của miền nghiệm là tam giác của hệ ba bất phương trình (một bất phương trình song song với trục toạ độ)</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>Diện tích miền nghiệm (tam giác) của hệ ba bất phương trình, một bất phương trình song song Ox hoặc Oy.</t>
+        </is>
+      </c>
+      <c r="L54" s="2" t="inlineStr">
+        <is>
+          <t>LUYEN TAP THEM - khong co trong yeu cau can dat cua Bo (dien tich mien nghiem la tam giac, he 3 bat phuong trinh co 1 bpt song song Ox hoac Oy). CLAUDE THEM 09/</t>
+        </is>
+      </c>
+      <c r="M54" s="2" t="inlineStr">
+        <is>
+          <t>Luyện tập thêm (ngoài YCCĐ)</t>
+        </is>
+      </c>
+      <c r="N54" s="2" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>B4</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>028</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>VD</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>SA</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>L10_C2_B4_VD028_SA_J</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H55" s="2" t="n"/>
+      <c r="I55" s="2" t="n"/>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>Diện tích và toạ độ đỉnh của miền nghiệm là tam giác của hệ ba bất phương trình (một bất phương trình song song với trục toạ độ)</t>
+        </is>
+      </c>
+      <c r="K55" s="2" t="inlineStr">
+        <is>
+          <t>Diện tích miền nghiệm (tam giác).</t>
+        </is>
+      </c>
+      <c r="L55" s="2" t="inlineStr">
+        <is>
+          <t>LUYEN TAP THEM - khong co trong yeu cau can dat cua Bo (dien tich mien nghiem la tam giac, he 3 bat phuong trinh co 1 bpt song song Ox hoac Oy). CLAUDE THEM 09/</t>
+        </is>
+      </c>
+      <c r="M55" s="2" t="inlineStr">
+        <is>
+          <t>Luyện tập thêm (ngoài YCCĐ)</t>
+        </is>
+      </c>
+      <c r="N55" s="2" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>B4</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>028</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>VD</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>MC</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>L10_C2_B4_VD028_MC_K</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>VDC</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="n"/>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
           <t>Tìm tham số m khi biết diện tích tam giác là miền nghiệm của hệ ba bất phương trình (bất phương trình song song với trục chứa tham số)</t>
         </is>
       </c>
-      <c r="K53" s="2" t="inlineStr">
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>Có tham số (VDC): biết diện tích tam giác, tìm m.</t>
+        </is>
+      </c>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>LUYEN TAP THEM - khong co trong yeu cau can dat cua Bo (dien tich mien nghiem la tam giac, he 3 bat phuong trinh co 1 bpt song song Ox hoac Oy). CLAUDE THEM 09/</t>
+        </is>
+      </c>
+      <c r="M56" s="2" t="inlineStr">
+        <is>
+          <t>muc_do_dang = VDC; Luyện tập thêm (ngoài YCCĐ)</t>
+        </is>
+      </c>
+      <c r="N56" s="2" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>B4</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>028</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>VD</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>SA</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>L10_C2_B4_VD028_SA_K</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>VDC</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="n"/>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>Tìm tham số m khi biết diện tích tam giác là miền nghiệm của hệ ba bất phương trình (bất phương trình song song với trục chứa tham số)</t>
+        </is>
+      </c>
+      <c r="K57" s="2" t="inlineStr">
+        <is>
+          <t>Có tham số (VDC): tìm m.</t>
+        </is>
+      </c>
+      <c r="L57" s="2" t="inlineStr">
+        <is>
+          <t>LUYEN TAP THEM - khong co trong yeu cau can dat cua Bo (dien tich mien nghiem la tam giac, he 3 bat phuong trinh co 1 bpt song song Ox hoac Oy). CLAUDE THEM 09/</t>
+        </is>
+      </c>
+      <c r="M57" s="2" t="inlineStr">
+        <is>
+          <t>muc_do_dang = VDC; Luyện tập thêm (ngoài YCCĐ)</t>
+        </is>
+      </c>
+      <c r="N57" s="2" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>B4</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>028</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>VD</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>L10_C2_B4_VD028_TL_F</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H58" s="2" t="n"/>
+      <c r="I58" s="2" t="n"/>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>Diện tích và toạ độ đỉnh của miền nghiệm là tam giác của hệ ba bất phương trình (một bất phương trình song song với trục toạ độ)</t>
+        </is>
+      </c>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>Tự luận 2 ý: a) toạ độ các đỉnh, b) diện tích tam giác miền nghiệm.</t>
+        </is>
+      </c>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>LUYEN TAP THEM - khong co trong yeu cau can dat cua Bo (dien tich mien nghiem la tam giac, he 3 bat phuong trinh co 1 bpt song song Ox hoac Oy). CLAUDE THEM 09/</t>
+        </is>
+      </c>
+      <c r="M58" s="2" t="inlineStr">
+        <is>
+          <t>Luyện tập thêm (ngoài YCCĐ)</t>
+        </is>
+      </c>
+      <c r="N58" s="2" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>B4</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>028</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>VD</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>L10_C2_B4_VD028_TL_G</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H59" s="2" t="n"/>
+      <c r="I59" s="2" t="n"/>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>Tìm tham số m khi biết diện tích tam giác là miền nghiệm của hệ ba bất phương trình (bất phương trình song song với trục chứa tham số)</t>
+        </is>
+      </c>
+      <c r="K59" s="2" t="inlineStr">
         <is>
           <t>Tự luận 2 ý có tham số: a) S theo m, b) cho S tìm m.</t>
         </is>
       </c>
-      <c r="L53" s="2" t="inlineStr">
+      <c r="L59" s="2" t="inlineStr">
         <is>
           <t>LUYEN TAP THEM - khong co trong yeu cau can dat cua Bo (dien tich mien nghiem la tam giac, he 3 bat phuong trinh co 1 bpt song song Ox hoac Oy). CLAUDE THEM 09/</t>
         </is>
       </c>
-      <c r="M53" s="3" t="inlineStr">
+      <c r="M59" s="2" t="inlineStr">
         <is>
           <t>Luyện tập thêm (ngoài YCCĐ)</t>
         </is>
       </c>
-      <c r="N53" s="2" t="inlineStr"/>
+      <c r="N59" s="2" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N53"/>
+  <autoFilter ref="A1:N59"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3545,7 +3913,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -3554,14 +3922,14 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Bảng ID Chương 2 lớp 10 (15/10/2026) - để cô đối chiếu; em CHƯA sửa gì ở Chương 2.</t>
+          <t>Bảng ID Chương 2 lớp 10 (cập nhật 15/10/2026 theo ID mới - dạng điểm thuộc miền nghiệm).</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Mỗi dòng là một ID trong data/mapping/toan10/L10_C2.json (đủ 52 ID, khớp đủ hàm Python).</t>
+          <t>Mỗi dòng là một ID trong data/mapping/toan10/L10_C2.json (đủ 58 ID, khớp đủ hàm Python).</t>
         </is>
       </c>
     </row>
@@ -3597,6 +3965,13 @@
       <c r="A7" t="inlineStr">
         <is>
           <t>Cột 'Cô ghi': cô ghi cách sửa (vd 'gộp B-I thành một chữ', 'giữ', 'tách kho bối cảnh'), em làm theo đợt sau.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>15/10/2026 đổi ID theo cô Lan: NB023_MC_A/SA_A -&gt; TH024_MC_B/SA_B; TH027_MC_B/SA_B (đa giác) -&gt; TH027_MC_C/SA_C; thêm NB024_MC_B/SA_B (hình 1 bpt), TH027_MC_B/SA_B (hình hệ), VD027_MC_B/SA_B (hệ, luyện tập thêm). Bảng đổi: data/mapping/doi_id/L10_C2_20261015_b.json.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
L10 C2 Bai 3: them muc VD - VD025 toan thuc te mot bat phuong trinh (MC_A, SA_A)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SrV2RdTxyMnQTjbX6LNoBV
</commit_message>
<xml_diff>
--- a/docs/bang_ID_L10_C2.xlsx
+++ b/docs/bang_ID_L10_C2.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Huong dan" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ID Chuong 2'!$A$1:$N$59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ID Chuong 2'!$A$1:$N$61</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N59"/>
+  <dimension ref="A1:N61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3176,12 +3176,12 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>B4</t>
+          <t>B3</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>028</t>
+          <t>025</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -3196,41 +3196,41 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>A</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_VD028_MC_H</t>
+          <t>L10_C2_B3_VD025_MC_A</t>
         </is>
       </c>
       <c r="G48" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H48" s="2" t="n"/>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>do_uong_an_kieng</t>
+          <t>thang_may, ve_xem_phim, quy_lop_lien_hoan, thu_vien_mua_sach</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>Bài toán thực tiễn đồ uống ăn kiêng: lập bất phương trình, hệ bất phương trình và tìm phương án có chi phí thấp nhất (calo và hai loại vitamin)</t>
+          <t>Toán thực tế: lập một bất phương trình bậc nhất hai ẩn từ tình huống, kết hợp điều kiện thêm (biết một ẩn, quan hệ giữa hai ẩn hoặc tổng số) để tìm giá trị nguyên lớn nhất</t>
         </is>
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>Tình huống 4 (VD): chọn hệ bất phương trình.</t>
+          <t>Trắc nghiệm cùng dạng với VD025_SA_A_01 (toán thực tế: giá trị nguyên lớn nhất thoả một bất phương trình bậc nhất hai ẩn và một điều kiện thêm). Nhiễu: lệch $1$, $2$ đơn vị và kết quả khi bỏ quên điều kiện thêm.</t>
         </is>
       </c>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 4); boi_canh do_uong_an_kieng; so lieu ngau nhien cung cau truc</t>
+          <t xml:space="preserve">CLAUDE THEM 15/10/2026 - co Lan duyet them VD025 (Bai 3 muc VD, de thuc te); MC goi lai SA_A voi dang=1; dap so chon truoc, so lieu suy nguoc; co Lan duyet lai </t>
         </is>
       </c>
       <c r="M48" s="2" t="inlineStr">
         <is>
-          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF; Cùng chữ "Dang" với các chữ H/I (MC/SA) của VD028: cùng dạng nhưng nhiều chữ (khác bối cảnh hoặc khác mức)</t>
+          <t>Mới 15/10/2026 (Bài 3 mức VD, đề thực tế; bối cảnh mới không trùng NB025/VD028/TF)</t>
         </is>
       </c>
       <c r="N48" s="2" t="n"/>
@@ -3238,12 +3238,12 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>B4</t>
+          <t>B3</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>028</t>
+          <t>025</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -3258,41 +3258,41 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>A</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_VD028_SA_H</t>
+          <t>L10_C2_B3_VD025_SA_A</t>
         </is>
       </c>
       <c r="G49" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H49" s="2" t="n"/>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>do_uong_an_kieng</t>
+          <t>thang_may, ve_xem_phim, quy_lop_lien_hoan, thu_vien_mua_sach</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr">
         <is>
-          <t>Bài toán thực tiễn đồ uống ăn kiêng: lập bất phương trình, hệ bất phương trình và tìm phương án có chi phí thấp nhất (calo và hai loại vitamin)</t>
+          <t>Toán thực tế: lập một bất phương trình bậc nhất hai ẩn từ tình huống, kết hợp điều kiện thêm (biết một ẩn, quan hệ giữa hai ẩn hoặc tổng số) để tìm giá trị nguyên lớn nhất</t>
         </is>
       </c>
       <c r="K49" s="2" t="inlineStr">
         <is>
-          <t>Tình huống 4 (VD): số đỉnh của miền nghiệm.</t>
+          <t xml:space="preserve">Toán thực tế (VD): lập MỘT bất phương trình bậc nhất hai ẩn từ tình huống, kết hợp điều kiện thêm (biết một ẩn, quan hệ giữa hai ẩn hoặc tổng số) để tìm giá trị nguyên lớn nhất. Bối cảnh: thang máy, vé xem phim, quỹ lớp </t>
         </is>
       </c>
       <c r="L49" s="2" t="inlineStr">
         <is>
-          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 4); boi_canh do_uong_an_kieng; so lieu ngau nhien cung cau truc</t>
+          <t>CLAUDE THEM 15/10/2026 - co Lan duyet them VD025 (Bai 3 muc VD, de thuc te); ban tra loi ngan cua VD025_MC_A (cung Dang); co Lan duyet lai noi dung</t>
         </is>
       </c>
       <c r="M49" s="2" t="inlineStr">
         <is>
-          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF; Cùng chữ "Dang" với các chữ H/I (MC/SA) của VD028: cùng dạng nhưng nhiều chữ (khác bối cảnh hoặc khác mức)</t>
+          <t>Mới 15/10/2026 (Bài 3 mức VD, đề thực tế; bối cảnh mới không trùng NB025/VD028/TF)</t>
         </is>
       </c>
       <c r="N49" s="2" t="n"/>
@@ -3320,22 +3320,18 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>H</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_VD028_MC_I</t>
+          <t>L10_C2_B4_VD028_MC_H</t>
         </is>
       </c>
       <c r="G50" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H50" s="2" t="inlineStr">
-        <is>
-          <t>VDC</t>
-        </is>
-      </c>
+      <c r="H50" s="2" t="n"/>
       <c r="I50" s="2" t="inlineStr">
         <is>
           <t>do_uong_an_kieng</t>
@@ -3348,7 +3344,7 @@
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>Tình huống 4 (VDC): giá trị tối ưu.</t>
+          <t>Tình huống 4 (VD): chọn hệ bất phương trình.</t>
         </is>
       </c>
       <c r="L50" s="2" t="inlineStr">
@@ -3358,7 +3354,7 @@
       </c>
       <c r="M50" s="2" t="inlineStr">
         <is>
-          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF; Cùng chữ "Dang" với các chữ H/I (MC/SA) của VD028: cùng dạng nhưng nhiều chữ (khác bối cảnh hoặc khác mức); muc_do_dang = VDC</t>
+          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF; Cùng chữ "Dang" với các chữ H/I (MC/SA) của VD028: cùng dạng nhưng nhiều chữ (khác bối cảnh hoặc khác mức)</t>
         </is>
       </c>
       <c r="N50" s="2" t="n"/>
@@ -3386,22 +3382,18 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>H</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_VD028_SA_I</t>
+          <t>L10_C2_B4_VD028_SA_H</t>
         </is>
       </c>
       <c r="G51" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H51" s="2" t="inlineStr">
-        <is>
-          <t>VDC</t>
-        </is>
-      </c>
+      <c r="H51" s="2" t="n"/>
       <c r="I51" s="2" t="inlineStr">
         <is>
           <t>do_uong_an_kieng</t>
@@ -3414,7 +3406,7 @@
       </c>
       <c r="K51" s="2" t="inlineStr">
         <is>
-          <t>Tình huống 4 (VDC): giá trị tối ưu.</t>
+          <t>Tình huống 4 (VD): số đỉnh của miền nghiệm.</t>
         </is>
       </c>
       <c r="L51" s="2" t="inlineStr">
@@ -3424,7 +3416,7 @@
       </c>
       <c r="M51" s="2" t="inlineStr">
         <is>
-          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF; Cùng chữ "Dang" với các chữ H/I (MC/SA) của VD028: cùng dạng nhưng nhiều chữ (khác bối cảnh hoặc khác mức); muc_do_dang = VDC</t>
+          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF; Cùng chữ "Dang" với các chữ H/I (MC/SA) của VD028: cùng dạng nhưng nhiều chữ (khác bối cảnh hoặc khác mức)</t>
         </is>
       </c>
       <c r="N51" s="2" t="n"/>
@@ -3447,23 +3439,27 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>TL</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>I</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_VD028_TL_E</t>
+          <t>L10_C2_B4_VD028_MC_I</t>
         </is>
       </c>
       <c r="G52" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H52" s="2" t="n"/>
+        <v>3</v>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>VDC</t>
+        </is>
+      </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
           <t>do_uong_an_kieng</t>
@@ -3476,7 +3472,7 @@
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>Tình huống 4: tự luận 2 ý (a lập hệ, b tối ưu).</t>
+          <t>Tình huống 4 (VDC): giá trị tối ưu.</t>
         </is>
       </c>
       <c r="L52" s="2" t="inlineStr">
@@ -3486,38 +3482,50 @@
       </c>
       <c r="M52" s="2" t="inlineStr">
         <is>
-          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF</t>
+          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF; Cùng chữ "Dang" với các chữ H/I (MC/SA) của VD028: cùng dạng nhưng nhiều chữ (khác bối cảnh hoặc khác mức); muc_do_dang = VDC</t>
         </is>
       </c>
       <c r="N52" s="2" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="n"/>
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>B4</t>
+        </is>
+      </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>(cả chương)</t>
-        </is>
-      </c>
-      <c r="C53" s="2" t="n"/>
+          <t>028</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>VD</t>
+        </is>
+      </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>TF</t>
+          <t>SA</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>I</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_TF_F</t>
+          <t>L10_C2_B4_VD028_SA_I</t>
         </is>
       </c>
       <c r="G53" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H53" s="2" t="n"/>
+        <v>3</v>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>VDC</t>
+        </is>
+      </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
           <t>do_uong_an_kieng</t>
@@ -3530,7 +3538,7 @@
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
-          <t>Tình huống 4: đúng/sai theo chương, bốn ý.</t>
+          <t>Tình huống 4 (VDC): giá trị tối ưu.</t>
         </is>
       </c>
       <c r="L53" s="2" t="inlineStr">
@@ -3540,7 +3548,7 @@
       </c>
       <c r="M53" s="2" t="inlineStr">
         <is>
-          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, 028</t>
+          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF; Cùng chữ "Dang" với các chữ H/I (MC/SA) của VD028: cùng dạng nhưng nhiều chữ (khác bối cảnh hoặc khác mức); muc_do_dang = VDC</t>
         </is>
       </c>
       <c r="N53" s="2" t="n"/>
@@ -3563,100 +3571,100 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>MC</t>
+          <t>TL</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>E</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_VD028_MC_J</t>
+          <t>L10_C2_B4_VD028_TL_E</t>
         </is>
       </c>
       <c r="G54" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H54" s="2" t="n"/>
-      <c r="I54" s="2" t="n"/>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>do_uong_an_kieng</t>
+        </is>
+      </c>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>Diện tích và toạ độ đỉnh của miền nghiệm là tam giác của hệ ba bất phương trình (một bất phương trình song song với trục toạ độ)</t>
+          <t>Bài toán thực tiễn đồ uống ăn kiêng: lập bất phương trình, hệ bất phương trình và tìm phương án có chi phí thấp nhất (calo và hai loại vitamin)</t>
         </is>
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>Diện tích miền nghiệm (tam giác) của hệ ba bất phương trình, một bất phương trình song song Ox hoặc Oy.</t>
+          <t>Tình huống 4: tự luận 2 ý (a lập hệ, b tối ưu).</t>
         </is>
       </c>
       <c r="L54" s="2" t="inlineStr">
         <is>
-          <t>LUYEN TAP THEM - khong co trong yeu cau can dat cua Bo (dien tich mien nghiem la tam giac, he 3 bat phuong trinh co 1 bpt song song Ox hoac Oy). CLAUDE THEM 09/</t>
+          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 4); boi_canh do_uong_an_kieng; so lieu ngau nhien cung cau truc</t>
         </is>
       </c>
       <c r="M54" s="2" t="inlineStr">
         <is>
-          <t>Luyện tập thêm (ngoài YCCĐ)</t>
+          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, TF</t>
         </is>
       </c>
       <c r="N54" s="2" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <t>B4</t>
-        </is>
-      </c>
+      <c r="A55" s="2" t="n"/>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>028</t>
-        </is>
-      </c>
-      <c r="C55" s="2" t="inlineStr">
-        <is>
-          <t>VD</t>
-        </is>
-      </c>
+          <t>(cả chương)</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="n"/>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>SA</t>
+          <t>TF</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>F</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_VD028_SA_J</t>
+          <t>L10_C2_TF_F</t>
         </is>
       </c>
       <c r="G55" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H55" s="2" t="n"/>
-      <c r="I55" s="2" t="n"/>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>do_uong_an_kieng</t>
+        </is>
+      </c>
       <c r="J55" s="2" t="inlineStr">
         <is>
-          <t>Diện tích và toạ độ đỉnh của miền nghiệm là tam giác của hệ ba bất phương trình (một bất phương trình song song với trục toạ độ)</t>
+          <t>Bài toán thực tiễn đồ uống ăn kiêng: lập bất phương trình, hệ bất phương trình và tìm phương án có chi phí thấp nhất (calo và hai loại vitamin)</t>
         </is>
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
-          <t>Diện tích miền nghiệm (tam giác).</t>
+          <t>Tình huống 4: đúng/sai theo chương, bốn ý.</t>
         </is>
       </c>
       <c r="L55" s="2" t="inlineStr">
         <is>
-          <t>LUYEN TAP THEM - khong co trong yeu cau can dat cua Bo (dien tich mien nghiem la tam giac, he 3 bat phuong trinh co 1 bpt song song Ox hoac Oy). CLAUDE THEM 09/</t>
+          <t>CLAUDE THEM 09/10/2026 - co Lan duyet (tinh huong thuc te 4); boi_canh do_uong_an_kieng; so lieu ngau nhien cung cau truc</t>
         </is>
       </c>
       <c r="M55" s="2" t="inlineStr">
         <is>
-          <t>Luyện tập thêm (ngoài YCCĐ)</t>
+          <t>Bối cảnh dùng chung với YCCĐ/TF khác: 025, 028</t>
         </is>
       </c>
       <c r="N55" s="2" t="n"/>
@@ -3684,31 +3692,27 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_VD028_MC_K</t>
+          <t>L10_C2_B4_VD028_MC_J</t>
         </is>
       </c>
       <c r="G56" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="H56" s="2" t="inlineStr">
-        <is>
-          <t>VDC</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="H56" s="2" t="n"/>
       <c r="I56" s="2" t="n"/>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>Tìm tham số m khi biết diện tích tam giác là miền nghiệm của hệ ba bất phương trình (bất phương trình song song với trục chứa tham số)</t>
+          <t>Diện tích và toạ độ đỉnh của miền nghiệm là tam giác của hệ ba bất phương trình (một bất phương trình song song với trục toạ độ)</t>
         </is>
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>Có tham số (VDC): biết diện tích tam giác, tìm m.</t>
+          <t>Diện tích miền nghiệm (tam giác) của hệ ba bất phương trình, một bất phương trình song song Ox hoặc Oy.</t>
         </is>
       </c>
       <c r="L56" s="2" t="inlineStr">
@@ -3718,7 +3722,7 @@
       </c>
       <c r="M56" s="2" t="inlineStr">
         <is>
-          <t>muc_do_dang = VDC; Luyện tập thêm (ngoài YCCĐ)</t>
+          <t>Luyện tập thêm (ngoài YCCĐ)</t>
         </is>
       </c>
       <c r="N56" s="2" t="n"/>
@@ -3746,31 +3750,27 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>J</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_VD028_SA_K</t>
+          <t>L10_C2_B4_VD028_SA_J</t>
         </is>
       </c>
       <c r="G57" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H57" s="2" t="inlineStr">
-        <is>
-          <t>VDC</t>
-        </is>
-      </c>
+      <c r="H57" s="2" t="n"/>
       <c r="I57" s="2" t="n"/>
       <c r="J57" s="2" t="inlineStr">
         <is>
-          <t>Tìm tham số m khi biết diện tích tam giác là miền nghiệm của hệ ba bất phương trình (bất phương trình song song với trục chứa tham số)</t>
+          <t>Diện tích và toạ độ đỉnh của miền nghiệm là tam giác của hệ ba bất phương trình (một bất phương trình song song với trục toạ độ)</t>
         </is>
       </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
-          <t>Có tham số (VDC): tìm m.</t>
+          <t>Diện tích miền nghiệm (tam giác).</t>
         </is>
       </c>
       <c r="L57" s="2" t="inlineStr">
@@ -3780,7 +3780,7 @@
       </c>
       <c r="M57" s="2" t="inlineStr">
         <is>
-          <t>muc_do_dang = VDC; Luyện tập thêm (ngoài YCCĐ)</t>
+          <t>Luyện tập thêm (ngoài YCCĐ)</t>
         </is>
       </c>
       <c r="N57" s="2" t="n"/>
@@ -3803,32 +3803,36 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>TL</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>K</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_VD028_TL_F</t>
+          <t>L10_C2_B4_VD028_MC_K</t>
         </is>
       </c>
       <c r="G58" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H58" s="2" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>VDC</t>
+        </is>
+      </c>
       <c r="I58" s="2" t="n"/>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>Diện tích và toạ độ đỉnh của miền nghiệm là tam giác của hệ ba bất phương trình (một bất phương trình song song với trục toạ độ)</t>
+          <t>Tìm tham số m khi biết diện tích tam giác là miền nghiệm của hệ ba bất phương trình (bất phương trình song song với trục chứa tham số)</t>
         </is>
       </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
-          <t>Tự luận 2 ý: a) toạ độ các đỉnh, b) diện tích tam giác miền nghiệm.</t>
+          <t>Có tham số (VDC): biết diện tích tam giác, tìm m.</t>
         </is>
       </c>
       <c r="L58" s="2" t="inlineStr">
@@ -3838,7 +3842,7 @@
       </c>
       <c r="M58" s="2" t="inlineStr">
         <is>
-          <t>Luyện tập thêm (ngoài YCCĐ)</t>
+          <t>muc_do_dang = VDC; Luyện tập thêm (ngoài YCCĐ)</t>
         </is>
       </c>
       <c r="N58" s="2" t="n"/>
@@ -3861,23 +3865,27 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>TL</t>
+          <t>SA</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>K</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>L10_C2_B4_VD028_TL_G</t>
+          <t>L10_C2_B4_VD028_SA_K</t>
         </is>
       </c>
       <c r="G59" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H59" s="2" t="n"/>
+        <v>2</v>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>VDC</t>
+        </is>
+      </c>
       <c r="I59" s="2" t="n"/>
       <c r="J59" s="2" t="inlineStr">
         <is>
@@ -3886,23 +3894,139 @@
       </c>
       <c r="K59" s="2" t="inlineStr">
         <is>
+          <t>Có tham số (VDC): tìm m.</t>
+        </is>
+      </c>
+      <c r="L59" s="2" t="inlineStr">
+        <is>
+          <t>LUYEN TAP THEM - khong co trong yeu cau can dat cua Bo (dien tich mien nghiem la tam giac, he 3 bat phuong trinh co 1 bpt song song Ox hoac Oy). CLAUDE THEM 09/</t>
+        </is>
+      </c>
+      <c r="M59" s="2" t="inlineStr">
+        <is>
+          <t>muc_do_dang = VDC; Luyện tập thêm (ngoài YCCĐ)</t>
+        </is>
+      </c>
+      <c r="N59" s="2" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>B4</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>028</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>VD</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>L10_C2_B4_VD028_TL_F</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H60" s="2" t="n"/>
+      <c r="I60" s="2" t="n"/>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>Diện tích và toạ độ đỉnh của miền nghiệm là tam giác của hệ ba bất phương trình (một bất phương trình song song với trục toạ độ)</t>
+        </is>
+      </c>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>Tự luận 2 ý: a) toạ độ các đỉnh, b) diện tích tam giác miền nghiệm.</t>
+        </is>
+      </c>
+      <c r="L60" s="2" t="inlineStr">
+        <is>
+          <t>LUYEN TAP THEM - khong co trong yeu cau can dat cua Bo (dien tich mien nghiem la tam giac, he 3 bat phuong trinh co 1 bpt song song Ox hoac Oy). CLAUDE THEM 09/</t>
+        </is>
+      </c>
+      <c r="M60" s="2" t="inlineStr">
+        <is>
+          <t>Luyện tập thêm (ngoài YCCĐ)</t>
+        </is>
+      </c>
+      <c r="N60" s="2" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>B4</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>028</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>VD</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>L10_C2_B4_VD028_TL_G</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H61" s="2" t="n"/>
+      <c r="I61" s="2" t="n"/>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>Tìm tham số m khi biết diện tích tam giác là miền nghiệm của hệ ba bất phương trình (bất phương trình song song với trục chứa tham số)</t>
+        </is>
+      </c>
+      <c r="K61" s="2" t="inlineStr">
+        <is>
           <t>Tự luận 2 ý có tham số: a) S theo m, b) cho S tìm m.</t>
         </is>
       </c>
-      <c r="L59" s="2" t="inlineStr">
+      <c r="L61" s="2" t="inlineStr">
         <is>
           <t>LUYEN TAP THEM - khong co trong yeu cau can dat cua Bo (dien tich mien nghiem la tam giac, he 3 bat phuong trinh co 1 bpt song song Ox hoac Oy). CLAUDE THEM 09/</t>
         </is>
       </c>
-      <c r="M59" s="2" t="inlineStr">
+      <c r="M61" s="2" t="inlineStr">
         <is>
           <t>Luyện tập thêm (ngoài YCCĐ)</t>
         </is>
       </c>
-      <c r="N59" s="2" t="n"/>
+      <c r="N61" s="2" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N59"/>
+  <autoFilter ref="A1:N61"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3913,7 +4037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -3929,7 +4053,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Mỗi dòng là một ID trong data/mapping/toan10/L10_C2.json (đủ 58 ID, khớp đủ hàm Python).</t>
+          <t>Mỗi dòng là một ID trong data/mapping/toan10/L10_C2.json (đủ 60 ID, khớp đủ hàm Python).</t>
         </is>
       </c>
     </row>
@@ -3972,6 +4096,13 @@
       <c r="A8" t="inlineStr">
         <is>
           <t>15/10/2026 đổi ID theo cô Lan: NB023_MC_A/SA_A -&gt; TH024_MC_B/SA_B; TH027_MC_B/SA_B (đa giác) -&gt; TH027_MC_C/SA_C; thêm NB024_MC_B/SA_B (hình 1 bpt), TH027_MC_B/SA_B (hình hệ), VD027_MC_B/SA_B (hệ, luyện tập thêm). Bảng đổi: data/mapping/doi_id/L10_C2_20261015_b.json.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>15/10/2026 thêm L10_C2_B3_VD025_MC_A/SA_A (Bài 3 mức VD, toán thực tế một bất phương trình; bối cảnh thang máy, vé xem phim, quỹ lớp liên hoan, thư viện mua sách).</t>
         </is>
       </c>
     </row>

</xml_diff>